<commit_message>
Roehampton: Related as partner on the whole estate, Grange at a £7m placeholder value
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFPSEueuEDo5NrLkRsAgfj
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -27,7 +27,7 @@
     <t xml:space="preserve">Roehampton Sports Ground Estate — underwrite model</t>
   </si>
   <si>
-    <t xml:space="preserve">Bruce Gillingham Pollard for Related · 17 October 2026 · Blue cells are inputs and match the BGP defaults on the appraisal page; everything else is a formula.</t>
+    <t xml:space="preserve">Bruce Gillingham Pollard with Related · 17 October 2026 · Blue cells are inputs and match the BGP defaults on the appraisal page; everything else is a formula.</t>
   </si>
   <si>
     <t xml:space="preserve">The bid</t>
@@ -147,13 +147,13 @@
     <t xml:space="preserve">Peppercorn to 2129</t>
   </si>
   <si>
-    <t xml:space="preserve">Year Related take The Grange</t>
+    <t xml:space="preserve">Year the Grange value is taken in</t>
   </si>
   <si>
     <t xml:space="preserve">year</t>
   </si>
   <si>
-    <t xml:space="preserve">0 = on completion; otherwise end of that year</t>
+    <t xml:space="preserve">Year the Grange value is taken in: 0 = on completion; otherwise end of that year</t>
   </si>
   <si>
     <t xml:space="preserve">Grange empty costs until then</t>
@@ -162,10 +162,10 @@
     <t xml:space="preserve">Service charge, rates, insurance</t>
   </si>
   <si>
-    <t xml:space="preserve">Grange price from Related</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per Woody Bruce, 17 October 2026</t>
+    <t xml:space="preserve">Grange value, placeholder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder value for The Grange pending Related's residential underwrite (Woody Bruce, 17 October 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Debt</t>
@@ -321,7 +321,7 @@
     <t xml:space="preserve">Cottages and Lodge</t>
   </si>
   <si>
-    <t xml:space="preserve">The Grange, to Related</t>
+    <t xml:space="preserve">The Grange, placeholder value</t>
   </si>
   <si>
     <t xml:space="preserve">Exit: Third Space, grounds and NTC reversion</t>

</xml_diff>

<commit_message>
Roehampton underwrite: single exit at the end of year 3, cottages and Grange sold with everything else
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFPSEueuEDo5NrLkRsAgfj
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="128">
   <si>
     <t xml:space="preserve">Roehampton Sports Ground Estate — underwrite model</t>
   </si>
@@ -138,7 +138,19 @@
     <t xml:space="preserve">Other lots</t>
   </si>
   <si>
-    <t xml:space="preserve">Cottages and Lodge, sold 2027</t>
+    <t xml:space="preserve">Cottages and Lodge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value of 1 and 2 Bank Lane and Clarence Lodge with vacant possession</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year the cottages are sold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 = on completion; otherwise end of that year. Everything is sold at once at the end of the hold.</t>
   </si>
   <si>
     <t xml:space="preserve">National Tennis Centre reversion at exit</t>
@@ -150,16 +162,13 @@
     <t xml:space="preserve">Year the Grange value is taken in</t>
   </si>
   <si>
-    <t xml:space="preserve">year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year the Grange value is taken in: 0 = on completion; otherwise end of that year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grange empty costs until then</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service charge, rates, insurance</t>
+    <t xml:space="preserve">Year the Grange value is taken in: 0 = on completion; otherwise end of that year. Everything is sold at once at the end of the hold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grange holding cost until sold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grange holding cost until sold: 0 while Related's underwrite carries the conversion costs and value; c. £1,000,000 pa if held empty</t>
   </si>
   <si>
     <t xml:space="preserve">Grange value, placeholder</t>
@@ -318,7 +327,7 @@
     <t xml:space="preserve">Rent received during the hold</t>
   </si>
   <si>
-    <t xml:space="preserve">Cottages and Lodge</t>
+    <t xml:space="preserve">Cottages and Lodge, at sale</t>
   </si>
   <si>
     <t xml:space="preserve">The Grange, placeholder value</t>
@@ -863,7 +872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1132,292 +1141,308 @@
       <c r="C23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="2"/>
+      <c r="D23" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="9" t="n">
-        <v>0.5</v>
+        <v>40</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>3</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25" s="8" t="n">
-        <v>0</v>
+        <v>43</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>0.5</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="8" t="n">
-        <v>1000000</v>
+        <v>3</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="D28" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>50</v>
-      </c>
+      <c r="A29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B30" s="7" t="n">
-        <v>0.07</v>
+        <v>0.55</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="2"/>
+      <c r="D30" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B31" s="7" t="n">
-        <v>0.015</v>
+        <v>0.07</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>0.55</v>
+        <v>0.015</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>55</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="D32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B33" s="7" t="n">
-        <v>0.06</v>
+        <v>0.55</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D33" s="2"/>
+      <c r="D33" s="3" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
+      <c r="A34" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>57</v>
-      </c>
+      <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="10" t="n">
+      <c r="A36" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="10" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$11</f>
         <v>1804260</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="10" t="n">
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="10" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
         <v>4510650</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B38" s="10" t="n">
-        <f aca="false">B37*Inputs!$B$16</f>
-        <v>676597.5</v>
-      </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B39" s="10" t="n">
-        <f aca="false">B36*Inputs!$B$13</f>
-        <v>1804260</v>
+        <f aca="false">B38*Inputs!$B$16</f>
+        <v>676597.5</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B40" s="10" t="n">
-        <f aca="false">B36*Inputs!$B$12</f>
-        <v>3608520</v>
+        <f aca="false">B37*Inputs!$B$13</f>
+        <v>1804260</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B41" s="10" t="n">
+        <f aca="false">B37*Inputs!$B$12</f>
+        <v>3608520</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B42" s="10" t="n">
         <f aca="false">Inputs!$B$5*1000000</f>
         <v>30000000</v>
       </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="10" t="n">
-        <f aca="false">Inputs!$B$27*1000000</f>
-        <v>7000000</v>
-      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B43" s="10" t="n">
+        <f aca="false">Inputs!$B$28*1000000</f>
+        <v>7000000</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B44" s="10" t="n">
         <f aca="false">Inputs!$B$23*1000000</f>
         <v>3000000</v>
       </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" s="10" t="n">
-        <f aca="false">Inputs!$B$24*1000000</f>
-        <v>500000</v>
-      </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B45" s="10" t="n">
-        <f aca="false">B36*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
-        <v>1804260</v>
+        <f aca="false">Inputs!$B$25*1000000</f>
+        <v>500000</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B46" s="11" t="n">
-        <f aca="false">MAX(0,Inputs!$B$12-(Inputs!$B$7-1))</f>
-        <v>0</v>
+        <v>70</v>
+      </c>
+      <c r="B46" s="10" t="n">
+        <f aca="false">B37*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
+        <v>1804260</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B47" s="10" t="n">
-        <f aca="false">B45/Inputs!$B$17/(1+Inputs!$B$6)-B46*B45</f>
-        <v>22525093.6329588</v>
+        <v>71</v>
+      </c>
+      <c r="B47" s="11" t="n">
+        <f aca="false">MAX(0,Inputs!$B$12-(Inputs!$B$7-1))</f>
+        <v>0</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B48" s="10" t="n">
+        <f aca="false">B46/Inputs!$B$17/(1+Inputs!$B$6)-B47*B46</f>
+        <v>22525093.6329588</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B49" s="10" t="n">
         <f aca="false">Inputs!$B$19/Inputs!$B$21/(1+Inputs!$B$6)</f>
         <v>1337613.69716426</v>
       </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1445,7 +1470,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1469,7 +1494,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1515,64 +1540,64 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="Q4" s="12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="R4" s="12" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="S4" s="12" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="T4" s="12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1592,48 +1617,48 @@
         <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">C5*IF(A5&lt;2,0,IF(A5-1&lt;=Inputs!$B$12,0,IF(A5-2&lt;Inputs!$B$12,A5-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A5-2)/5))))</f>
+        <f aca="false">C5*IF(A5&lt;2,0,IF(A5-1&lt;=Inputs!$B$12,0,IF(A5-2&lt;Inputs!$B$12,A5-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A5-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A5=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A5=Inputs!$B$25),Inputs!$B$42,0))</f>
-        <v>7000000</v>
+        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A5=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A5=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <f aca="false">-C5*(IF(A5=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A5=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A5=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C5*(IF(A5=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A5=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A5=2,Inputs!$B$40,0))</f>
         <v>-32040000</v>
       </c>
       <c r="H5" s="10" t="n">
-        <f aca="false">-C5*IF(AND(Inputs!$B$25&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C5*IF(AND(Inputs!$B$26&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I5" s="10" t="n">
-        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">SUM(D5:I5)</f>
-        <v>-25040000</v>
+        <v>-32040000</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">-G5-F5</f>
-        <v>25040000</v>
+        <v>32040000</v>
       </c>
       <c r="L5" s="10" t="n">
-        <f aca="false">IF(K5&gt;0,Inputs!$B$29*K5,0)</f>
-        <v>13772000</v>
+        <f aca="false">IF(K5&gt;0,Inputs!$B$30*K5,0)</f>
+        <v>17622000</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="N5" s="10" t="n">
-        <f aca="false">M5*Inputs!$B$30</f>
+        <f aca="false">M5*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O5" s="10" t="n">
-        <f aca="false">L5*Inputs!$B$31</f>
-        <v>206580</v>
+        <f aca="false">L5*Inputs!$B$32</f>
+        <v>264330</v>
       </c>
       <c r="P5" s="10" t="n">
         <f aca="false">IF(K5&lt;0,MIN(M5+L5,-K5),0)+IF(A5=Inputs!$B$7,M5+L5-IF(K5&lt;0,MIN(M5+L5,-K5),0),0)</f>
@@ -1641,19 +1666,19 @@
       </c>
       <c r="Q5" s="10" t="n">
         <f aca="false">M5+L5-P5</f>
-        <v>13772000</v>
+        <v>17622000</v>
       </c>
       <c r="R5" s="10" t="n">
         <f aca="false">L5-N5-P5-O5</f>
-        <v>13565420</v>
+        <v>17357670</v>
       </c>
       <c r="S5" s="10" t="n">
         <f aca="false">J5+R5</f>
-        <v>-11474580</v>
+        <v>-14682330</v>
       </c>
       <c r="T5" s="10" t="n">
         <f aca="false">S5</f>
-        <v>-11474580</v>
+        <v>-14682330</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,48 +1698,48 @@
         <v>350000</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">C6*IF(A6&lt;2,0,IF(A6-1&lt;=Inputs!$B$12,0,IF(A6-2&lt;Inputs!$B$12,A6-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A6-2)/5))))</f>
+        <f aca="false">C6*IF(A6&lt;2,0,IF(A6-1&lt;=Inputs!$B$12,0,IF(A6-2&lt;Inputs!$B$12,A6-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A6-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A6=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A6=Inputs!$B$25),Inputs!$B$42,0))</f>
-        <v>3000000</v>
+        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A6=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A6=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">-C6*(IF(A6=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A6=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A6=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C6*(IF(A6=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A6=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A6=2,Inputs!$B$40,0))</f>
         <v>-5187247.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <f aca="false">-C6*IF(AND(Inputs!$B$25&gt;0,A6&gt;=1,A6&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C6*IF(AND(Inputs!$B$26&gt;0,A6&gt;=1,A6&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="10" t="n">
         <f aca="false">SUM(D6:I6)</f>
-        <v>-1837247.5</v>
+        <v>-4837247.5</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">-G6-F6</f>
-        <v>2187247.5</v>
+        <v>5187247.5</v>
       </c>
       <c r="L6" s="10" t="n">
-        <f aca="false">IF(K6&gt;0,Inputs!$B$29*K6,0)</f>
-        <v>1202986.125</v>
+        <f aca="false">IF(K6&gt;0,Inputs!$B$30*K6,0)</f>
+        <v>2852986.125</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">Q5</f>
-        <v>13772000</v>
+        <v>17622000</v>
       </c>
       <c r="N6" s="10" t="n">
-        <f aca="false">M6*Inputs!$B$30</f>
-        <v>964040</v>
+        <f aca="false">M6*Inputs!$B$31</f>
+        <v>1233540</v>
       </c>
       <c r="O6" s="10" t="n">
-        <f aca="false">L6*Inputs!$B$31</f>
-        <v>18044.791875</v>
+        <f aca="false">L6*Inputs!$B$32</f>
+        <v>42794.791875</v>
       </c>
       <c r="P6" s="10" t="n">
         <f aca="false">IF(K6&lt;0,MIN(M6+L6,-K6),0)+IF(A6=Inputs!$B$7,M6+L6-IF(K6&lt;0,MIN(M6+L6,-K6),0),0)</f>
@@ -1722,19 +1747,19 @@
       </c>
       <c r="Q6" s="10" t="n">
         <f aca="false">M6+L6-P6</f>
-        <v>14974986.125</v>
+        <v>20474986.125</v>
       </c>
       <c r="R6" s="10" t="n">
         <f aca="false">L6-N6-P6-O6</f>
-        <v>220901.333125</v>
+        <v>1576651.333125</v>
       </c>
       <c r="S6" s="10" t="n">
         <f aca="false">J6+R6</f>
-        <v>-1616346.166875</v>
+        <v>-3260596.166875</v>
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">T5+S6</f>
-        <v>-13090926.166875</v>
+        <v>-17942926.166875</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1754,23 +1779,23 @@
         <v>100000</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">C7*IF(A7&lt;2,0,IF(A7-1&lt;=Inputs!$B$12,0,IF(A7-2&lt;Inputs!$B$12,A7-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A7-2)/5))))</f>
+        <f aca="false">C7*IF(A7&lt;2,0,IF(A7-1&lt;=Inputs!$B$12,0,IF(A7-2&lt;Inputs!$B$12,A7-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A7-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A7=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A7=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A7=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A7=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
-        <f aca="false">-C7*(IF(A7=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A7=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A7=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C7*(IF(A7=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A7=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A7=2,Inputs!$B$40,0))</f>
         <v>-1804260</v>
       </c>
       <c r="H7" s="10" t="n">
-        <f aca="false">-C7*IF(AND(Inputs!$B$25&gt;0,A7&gt;=1,A7&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C7*IF(AND(Inputs!$B$26&gt;0,A7&gt;=1,A7&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I7" s="10" t="n">
-        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="10" t="n">
@@ -1782,19 +1807,19 @@
         <v>1804260</v>
       </c>
       <c r="L7" s="10" t="n">
-        <f aca="false">IF(K7&gt;0,Inputs!$B$29*K7,0)</f>
+        <f aca="false">IF(K7&gt;0,Inputs!$B$30*K7,0)</f>
         <v>992343</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">Q6</f>
-        <v>14974986.125</v>
+        <v>20474986.125</v>
       </c>
       <c r="N7" s="10" t="n">
-        <f aca="false">M7*Inputs!$B$30</f>
-        <v>1048249.02875</v>
+        <f aca="false">M7*Inputs!$B$31</f>
+        <v>1433249.02875</v>
       </c>
       <c r="O7" s="10" t="n">
-        <f aca="false">L7*Inputs!$B$31</f>
+        <f aca="false">L7*Inputs!$B$32</f>
         <v>14885.145</v>
       </c>
       <c r="P7" s="10" t="n">
@@ -1803,19 +1828,19 @@
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">M7+L7-P7</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
       <c r="R7" s="10" t="n">
         <f aca="false">L7-N7-P7-O7</f>
-        <v>-70791.1737500001</v>
+        <v>-455791.17375</v>
       </c>
       <c r="S7" s="10" t="n">
         <f aca="false">J7+R7</f>
-        <v>-1775051.17375</v>
+        <v>-2160051.17375</v>
       </c>
       <c r="T7" s="10" t="n">
         <f aca="false">T6+S7</f>
-        <v>-14865977.340625</v>
+        <v>-20102977.340625</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,52 +1860,52 @@
         <v>100000</v>
       </c>
       <c r="E8" s="10" t="n">
-        <f aca="false">C8*IF(A8&lt;2,0,IF(A8-1&lt;=Inputs!$B$12,0,IF(A8-2&lt;Inputs!$B$12,A8-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A8-2)/5))))</f>
+        <f aca="false">C8*IF(A8&lt;2,0,IF(A8-1&lt;=Inputs!$B$12,0,IF(A8-2&lt;Inputs!$B$12,A8-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A8-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F8" s="10" t="n">
-        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A8=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A8=Inputs!$B$25),Inputs!$B$42,0))</f>
-        <v>0</v>
+        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A8=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A8=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <v>10000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <f aca="false">-C8*(IF(A8=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A8=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A8=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C8*(IF(A8=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A8=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A8=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H8" s="10" t="n">
-        <f aca="false">-C8*IF(AND(Inputs!$B$25&gt;0,A8&gt;=1,A8&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C8*IF(AND(Inputs!$B$26&gt;0,A8&gt;=1,A8&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>24362707.3301231</v>
       </c>
       <c r="J8" s="10" t="n">
         <f aca="false">SUM(D8:I8)</f>
-        <v>24462707.3301231</v>
+        <v>34462707.3301231</v>
       </c>
       <c r="K8" s="10" t="n">
         <f aca="false">-G8-F8</f>
-        <v>0</v>
+        <v>-10000000</v>
       </c>
       <c r="L8" s="10" t="n">
-        <f aca="false">IF(K8&gt;0,Inputs!$B$29*K8,0)</f>
+        <f aca="false">IF(K8&gt;0,Inputs!$B$30*K8,0)</f>
         <v>0</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">Q7</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
       <c r="N8" s="10" t="n">
-        <f aca="false">M8*Inputs!$B$30</f>
-        <v>1117713.03875</v>
+        <f aca="false">M8*Inputs!$B$31</f>
+        <v>1502713.03875</v>
       </c>
       <c r="O8" s="10" t="n">
-        <f aca="false">L8*Inputs!$B$31</f>
+        <f aca="false">L8*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P8" s="10" t="n">
         <f aca="false">IF(K8&lt;0,MIN(M8+L8,-K8),0)+IF(A8=Inputs!$B$7,M8+L8-IF(K8&lt;0,MIN(M8+L8,-K8),0),0)</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
       <c r="Q8" s="10" t="n">
         <f aca="false">M8+L8-P8</f>
@@ -1888,15 +1913,15 @@
       </c>
       <c r="R8" s="10" t="n">
         <f aca="false">L8-N8-P8-O8</f>
-        <v>-17085042.16375</v>
+        <v>-22970042.16375</v>
       </c>
       <c r="S8" s="10" t="n">
         <f aca="false">J8+R8</f>
-        <v>7377665.16637306</v>
+        <v>11492665.1663731</v>
       </c>
       <c r="T8" s="10" t="n">
         <f aca="false">T7+S8</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1916,23 +1941,23 @@
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <f aca="false">C9*IF(A9&lt;2,0,IF(A9-1&lt;=Inputs!$B$12,0,IF(A9-2&lt;Inputs!$B$12,A9-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A9-2)/5))))</f>
+        <f aca="false">C9*IF(A9&lt;2,0,IF(A9-1&lt;=Inputs!$B$12,0,IF(A9-2&lt;Inputs!$B$12,A9-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A9-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
-        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A9=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A9=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A9=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A9=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
-        <f aca="false">-C9*(IF(A9=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A9=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A9=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C9*(IF(A9=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A9=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A9=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H9" s="10" t="n">
-        <f aca="false">-C9*IF(AND(Inputs!$B$25&gt;0,A9&gt;=1,A9&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C9*IF(AND(Inputs!$B$26&gt;0,A9&gt;=1,A9&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I9" s="10" t="n">
-        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="10" t="n">
@@ -1944,7 +1969,7 @@
         <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <f aca="false">IF(K9&gt;0,Inputs!$B$29*K9,0)</f>
+        <f aca="false">IF(K9&gt;0,Inputs!$B$30*K9,0)</f>
         <v>0</v>
       </c>
       <c r="M9" s="10" t="n">
@@ -1952,11 +1977,11 @@
         <v>0</v>
       </c>
       <c r="N9" s="10" t="n">
-        <f aca="false">M9*Inputs!$B$30</f>
+        <f aca="false">M9*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O9" s="10" t="n">
-        <f aca="false">L9*Inputs!$B$31</f>
+        <f aca="false">L9*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P9" s="10" t="n">
@@ -1977,7 +2002,7 @@
       </c>
       <c r="T9" s="10" t="n">
         <f aca="false">T8+S9</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1997,23 +2022,23 @@
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <f aca="false">C10*IF(A10&lt;2,0,IF(A10-1&lt;=Inputs!$B$12,0,IF(A10-2&lt;Inputs!$B$12,A10-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A10-2)/5))))</f>
+        <f aca="false">C10*IF(A10&lt;2,0,IF(A10-1&lt;=Inputs!$B$12,0,IF(A10-2&lt;Inputs!$B$12,A10-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A10-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A10=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A10=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A10=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A10=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <f aca="false">-C10*(IF(A10=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A10=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A10=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C10*(IF(A10=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A10=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A10=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H10" s="10" t="n">
-        <f aca="false">-C10*IF(AND(Inputs!$B$25&gt;0,A10&gt;=1,A10&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C10*IF(AND(Inputs!$B$26&gt;0,A10&gt;=1,A10&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J10" s="10" t="n">
@@ -2025,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="L10" s="10" t="n">
-        <f aca="false">IF(K10&gt;0,Inputs!$B$29*K10,0)</f>
+        <f aca="false">IF(K10&gt;0,Inputs!$B$30*K10,0)</f>
         <v>0</v>
       </c>
       <c r="M10" s="10" t="n">
@@ -2033,11 +2058,11 @@
         <v>0</v>
       </c>
       <c r="N10" s="10" t="n">
-        <f aca="false">M10*Inputs!$B$30</f>
+        <f aca="false">M10*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O10" s="10" t="n">
-        <f aca="false">L10*Inputs!$B$31</f>
+        <f aca="false">L10*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P10" s="10" t="n">
@@ -2058,7 +2083,7 @@
       </c>
       <c r="T10" s="10" t="n">
         <f aca="false">T9+S10</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2078,23 +2103,23 @@
         <v>0</v>
       </c>
       <c r="E11" s="10" t="n">
-        <f aca="false">C11*IF(A11&lt;2,0,IF(A11-1&lt;=Inputs!$B$12,0,IF(A11-2&lt;Inputs!$B$12,A11-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A11-2)/5))))</f>
+        <f aca="false">C11*IF(A11&lt;2,0,IF(A11-1&lt;=Inputs!$B$12,0,IF(A11-2&lt;Inputs!$B$12,A11-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A11-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F11" s="10" t="n">
-        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A11=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A11=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A11=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A11=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <f aca="false">-C11*(IF(A11=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A11=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A11=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C11*(IF(A11=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A11=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A11=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H11" s="10" t="n">
-        <f aca="false">-C11*IF(AND(Inputs!$B$25&gt;0,A11&gt;=1,A11&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C11*IF(AND(Inputs!$B$26&gt;0,A11&gt;=1,A11&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="10" t="n">
@@ -2106,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
-        <f aca="false">IF(K11&gt;0,Inputs!$B$29*K11,0)</f>
+        <f aca="false">IF(K11&gt;0,Inputs!$B$30*K11,0)</f>
         <v>0</v>
       </c>
       <c r="M11" s="10" t="n">
@@ -2114,11 +2139,11 @@
         <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
-        <f aca="false">M11*Inputs!$B$30</f>
+        <f aca="false">M11*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O11" s="10" t="n">
-        <f aca="false">L11*Inputs!$B$31</f>
+        <f aca="false">L11*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P11" s="10" t="n">
@@ -2139,7 +2164,7 @@
       </c>
       <c r="T11" s="10" t="n">
         <f aca="false">T10+S11</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2159,23 +2184,23 @@
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <f aca="false">C12*IF(A12&lt;2,0,IF(A12-1&lt;=Inputs!$B$12,0,IF(A12-2&lt;Inputs!$B$12,A12-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A12-2)/5))))</f>
+        <f aca="false">C12*IF(A12&lt;2,0,IF(A12-1&lt;=Inputs!$B$12,0,IF(A12-2&lt;Inputs!$B$12,A12-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A12-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A12=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A12=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A12=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A12=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
-        <f aca="false">-C12*(IF(A12=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A12=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A12=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C12*(IF(A12=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A12=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A12=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H12" s="10" t="n">
-        <f aca="false">-C12*IF(AND(Inputs!$B$25&gt;0,A12&gt;=1,A12&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C12*IF(AND(Inputs!$B$26&gt;0,A12&gt;=1,A12&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J12" s="10" t="n">
@@ -2187,7 +2212,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="10" t="n">
-        <f aca="false">IF(K12&gt;0,Inputs!$B$29*K12,0)</f>
+        <f aca="false">IF(K12&gt;0,Inputs!$B$30*K12,0)</f>
         <v>0</v>
       </c>
       <c r="M12" s="10" t="n">
@@ -2195,11 +2220,11 @@
         <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
-        <f aca="false">M12*Inputs!$B$30</f>
+        <f aca="false">M12*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O12" s="10" t="n">
-        <f aca="false">L12*Inputs!$B$31</f>
+        <f aca="false">L12*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P12" s="10" t="n">
@@ -2220,7 +2245,7 @@
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">T11+S12</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,23 +2265,23 @@
         <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">C13*IF(A13&lt;2,0,IF(A13-1&lt;=Inputs!$B$12,0,IF(A13-2&lt;Inputs!$B$12,A13-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A13-2)/5))))</f>
+        <f aca="false">C13*IF(A13&lt;2,0,IF(A13-1&lt;=Inputs!$B$12,0,IF(A13-2&lt;Inputs!$B$12,A13-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A13-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A13=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A13=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A13=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A13=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
-        <f aca="false">-C13*(IF(A13=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A13=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A13=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C13*(IF(A13=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A13=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A13=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H13" s="10" t="n">
-        <f aca="false">-C13*IF(AND(Inputs!$B$25&gt;0,A13&gt;=1,A13&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C13*IF(AND(Inputs!$B$26&gt;0,A13&gt;=1,A13&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I13" s="10" t="n">
-        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="10" t="n">
@@ -2268,7 +2293,7 @@
         <v>0</v>
       </c>
       <c r="L13" s="10" t="n">
-        <f aca="false">IF(K13&gt;0,Inputs!$B$29*K13,0)</f>
+        <f aca="false">IF(K13&gt;0,Inputs!$B$30*K13,0)</f>
         <v>0</v>
       </c>
       <c r="M13" s="10" t="n">
@@ -2276,11 +2301,11 @@
         <v>0</v>
       </c>
       <c r="N13" s="10" t="n">
-        <f aca="false">M13*Inputs!$B$30</f>
+        <f aca="false">M13*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O13" s="10" t="n">
-        <f aca="false">L13*Inputs!$B$31</f>
+        <f aca="false">L13*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P13" s="10" t="n">
@@ -2301,7 +2326,7 @@
       </c>
       <c r="T13" s="10" t="n">
         <f aca="false">T12+S13</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,23 +2346,23 @@
         <v>0</v>
       </c>
       <c r="E14" s="10" t="n">
-        <f aca="false">C14*IF(A14&lt;2,0,IF(A14-1&lt;=Inputs!$B$12,0,IF(A14-2&lt;Inputs!$B$12,A14-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A14-2)/5))))</f>
+        <f aca="false">C14*IF(A14&lt;2,0,IF(A14-1&lt;=Inputs!$B$12,0,IF(A14-2&lt;Inputs!$B$12,A14-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A14-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
-        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A14=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A14=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A14=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A14=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
-        <f aca="false">-C14*(IF(A14=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A14=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A14=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C14*(IF(A14=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A14=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A14=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H14" s="10" t="n">
-        <f aca="false">-C14*IF(AND(Inputs!$B$25&gt;0,A14&gt;=1,A14&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C14*IF(AND(Inputs!$B$26&gt;0,A14&gt;=1,A14&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J14" s="10" t="n">
@@ -2349,7 +2374,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="10" t="n">
-        <f aca="false">IF(K14&gt;0,Inputs!$B$29*K14,0)</f>
+        <f aca="false">IF(K14&gt;0,Inputs!$B$30*K14,0)</f>
         <v>0</v>
       </c>
       <c r="M14" s="10" t="n">
@@ -2357,11 +2382,11 @@
         <v>0</v>
       </c>
       <c r="N14" s="10" t="n">
-        <f aca="false">M14*Inputs!$B$30</f>
+        <f aca="false">M14*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O14" s="10" t="n">
-        <f aca="false">L14*Inputs!$B$31</f>
+        <f aca="false">L14*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P14" s="10" t="n">
@@ -2382,7 +2407,7 @@
       </c>
       <c r="T14" s="10" t="n">
         <f aca="false">T13+S14</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2402,23 +2427,23 @@
         <v>0</v>
       </c>
       <c r="E15" s="10" t="n">
-        <f aca="false">C15*IF(A15&lt;2,0,IF(A15-1&lt;=Inputs!$B$12,0,IF(A15-2&lt;Inputs!$B$12,A15-1-Inputs!$B$12,1)*Inputs!$B$36*(1+Inputs!$B$14)^(5*INT((A15-2)/5))))</f>
+        <f aca="false">C15*IF(A15&lt;2,0,IF(A15-1&lt;=Inputs!$B$12,0,IF(A15-2&lt;Inputs!$B$12,A15-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A15-2)/5))))</f>
         <v>0</v>
       </c>
       <c r="F15" s="10" t="n">
-        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$25=0,Inputs!$B$42,0),0)+IF(A15=1,Inputs!$B$43,0)+IF(AND(Inputs!$B$25&gt;0,A15=Inputs!$B$25),Inputs!$B$42,0))</f>
+        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A15=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A15=Inputs!$B$26),Inputs!$B$43,0))</f>
         <v>0</v>
       </c>
       <c r="G15" s="10" t="n">
-        <f aca="false">-C15*(IF(A15=0,Inputs!$B$41*(1+Inputs!$B$6),0)+IF(A15=1,Inputs!$B$37+Inputs!$B$38+Inputs!$B$20,0)+IF(A15=2,Inputs!$B$39,0))</f>
+        <f aca="false">-C15*(IF(A15=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A15=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A15=2,Inputs!$B$40,0))</f>
         <v>-0</v>
       </c>
       <c r="H15" s="10" t="n">
-        <f aca="false">-C15*IF(AND(Inputs!$B$25&gt;0,A15&gt;=1,A15&lt;=Inputs!$B$25),Inputs!$B$26,0)</f>
+        <f aca="false">-C15*IF(AND(Inputs!$B$26&gt;0,A15&gt;=1,A15&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
         <v>-0</v>
       </c>
       <c r="I15" s="10" t="n">
-        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$47+Inputs!$B$48+Inputs!$B$44,0)</f>
+        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
         <v>0</v>
       </c>
       <c r="J15" s="10" t="n">
@@ -2430,7 +2455,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="10" t="n">
-        <f aca="false">IF(K15&gt;0,Inputs!$B$29*K15,0)</f>
+        <f aca="false">IF(K15&gt;0,Inputs!$B$30*K15,0)</f>
         <v>0</v>
       </c>
       <c r="M15" s="10" t="n">
@@ -2438,11 +2463,11 @@
         <v>0</v>
       </c>
       <c r="N15" s="10" t="n">
-        <f aca="false">M15*Inputs!$B$30</f>
+        <f aca="false">M15*Inputs!$B$31</f>
         <v>0</v>
       </c>
       <c r="O15" s="10" t="n">
-        <f aca="false">L15*Inputs!$B$31</f>
+        <f aca="false">L15*Inputs!$B$32</f>
         <v>0</v>
       </c>
       <c r="P15" s="10" t="n">
@@ -2463,13 +2488,13 @@
       </c>
       <c r="T15" s="10" t="n">
         <f aca="false">T14+S15</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="13" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="14" t="n">
@@ -2506,35 +2531,35 @@
       </c>
       <c r="L16" s="14" t="n">
         <f aca="false">SUM(L5:L15)</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
       <c r="M16" s="14" t="n">
         <f aca="false">SUM(M5:M15)</f>
-        <v>44714315.25</v>
+        <v>59564315.25</v>
       </c>
       <c r="N16" s="14" t="n">
         <f aca="false">SUM(N5:N15)</f>
-        <v>3130002.0675</v>
+        <v>4169502.0675</v>
       </c>
       <c r="O16" s="14" t="n">
         <f aca="false">SUM(O5:O15)</f>
-        <v>239509.936875</v>
+        <v>322009.936875</v>
       </c>
       <c r="P16" s="14" t="n">
         <f aca="false">SUM(P5:P15)</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
       <c r="Q16" s="14" t="n">
         <f aca="false">SUM(Q5:Q15)</f>
-        <v>44714315.25</v>
+        <v>59564315.25</v>
       </c>
       <c r="R16" s="14" t="n">
         <f aca="false">SUM(R5:R15)</f>
-        <v>-3369512.004375</v>
+        <v>-4491512.004375</v>
       </c>
       <c r="S16" s="14" t="n">
         <f aca="false">SUM(S5:S15)</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
       <c r="T16" s="2"/>
     </row>
@@ -2563,13 +2588,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2"/>
     </row>
@@ -2579,13 +2604,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">'Cash flow'!D16+'Cash flow'!E16</f>
@@ -2594,25 +2619,25 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">Inputs!$B$43</f>
+        <f aca="false">Inputs!$B$44</f>
         <v>3000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">Inputs!$B$42</f>
+        <f aca="false">Inputs!$B$43</f>
         <v>7000000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B8" s="10" t="n">
         <f aca="false">'Cash flow'!I16</f>
@@ -2621,7 +2646,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -2630,13 +2655,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">-'Cash flow'!G16-'Cash flow'!H16</f>
@@ -2645,184 +2670,184 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">'Cash flow'!N16+'Cash flow'!O16</f>
-        <v>3369512.004375</v>
+        <v>4491512.004375</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B13" s="10" t="n">
         <f aca="false">B11+B12</f>
-        <v>42401019.504375</v>
+        <v>43523019.504375</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B14" s="15" t="n">
         <f aca="false">(B9-B13)/B13</f>
-        <v>-0.176606889687624</v>
+        <v>-0.19783352056689</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">B9-B13</f>
-        <v>-7488312.17425194</v>
+        <v>-8610312.17425194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">B16/B9</f>
-        <v>-0.214486722655019</v>
+        <v>-0.246624018379201</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B18" s="15" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$19)/(B11-Inputs!$B$42-Inputs!$B$43)</f>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/(B11-Inputs!$B$43-Inputs!$B$44)</f>
         <v>0.0655928735357611</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B19" s="15" t="n">
         <f aca="false">IRR('Cash flow'!J5:J15)</f>
-        <v>-0.0538941068036766</v>
+        <v>-0.0397824334770132</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B20" s="15" t="n">
         <f aca="false">IRR('Cash flow'!S5:S15)</f>
-        <v>-0.237603166499829</v>
+        <v>-0.195509552228641</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
-        <v>0.496278515520923</v>
+        <v>0.571689704049368</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B22" s="10" t="n">
         <f aca="false">-MIN('Cash flow'!T5:T15)</f>
-        <v>14865977.340625</v>
+        <v>20102977.340625</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">MAX('Cash flow'!Q5:Q15)</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B24" s="15" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$19-B23*Inputs!$B$30)/B22</f>
-        <v>0.05290919952505</v>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$19-B23*Inputs!$B$31)/B22</f>
+        <v>0.0199745020076472</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B26" s="10" t="n">
-        <f aca="false">(Inputs!$B$36/Inputs!$B$17+Inputs!$B$19/Inputs!$B$21)/(1+Inputs!$B$6)+Inputs!$B$44</f>
+        <f aca="false">(Inputs!$B$37/Inputs!$B$17+Inputs!$B$19/Inputs!$B$21)/(1+Inputs!$B$6)+Inputs!$B$45</f>
         <v>24362707.3301231</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">'Cash flow'!Q7</f>
-        <v>15967329.125</v>
+        <v>21467329.125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B28" s="10" t="n">
-        <f aca="false">B26*Inputs!$B$32</f>
+        <f aca="false">B26*Inputs!$B$33</f>
         <v>13399489.0315677</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B29" s="10" t="n">
         <f aca="false">B28-B27</f>
-        <v>-2567840.09343232</v>
+        <v>-8067840.09343232</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B30" s="15" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$19)/B28</f>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/B28</f>
         <v>0.142114374325303</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B31" s="16" t="n">
-        <f aca="false">(Inputs!$B$36+Inputs!$B$19)/(B28*Inputs!$B$33)</f>
+        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/(B28*Inputs!$B$34)</f>
         <v>2.36857290542172</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B32" s="10" t="n">
-        <f aca="false">MAX(0,(B28*Inputs!$B$33-Inputs!$B$19)*Inputs!$B$12)</f>
+        <f aca="false">MAX(0,(B28*Inputs!$B$34-Inputs!$B$19)*Inputs!$B$12)</f>
         <v>1407938.68378812</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Roehampton: same-day completion of purchase, Third Space lease and Club regrant; no landlord's works; Excel model fixed
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="121">
   <si>
     <t xml:space="preserve">Roehampton Sports Ground Estate — underwrite model</t>
   </si>
@@ -39,7 +39,7 @@
     <t xml:space="preserve">£m</t>
   </si>
   <si>
-    <t xml:space="preserve">Working price; no guide published. The appraisal page gives c. £20m for 15% on cost with The Grange at £7m. Use Goal Seek: set Outputs!B13 to 0.15 by changing Inputs!B5.</t>
+    <t xml:space="preserve">Working price; no guide published. The appraisal page gives the bid for 15% on cost with the residential placeholder at £7m. Use Goal Seek on Outputs, Profit on cost, by changing this cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Purchaser's costs</t>
@@ -105,7 +105,7 @@
     <t xml:space="preserve">£ psf</t>
   </si>
   <si>
-    <t xml:space="preserve">Base build and separation; tenant fits out</t>
+    <t xml:space="preserve">Nil: Third Space fit out from the capital contribution and nothing more is spent on the leisure side</t>
   </si>
   <si>
     <t xml:space="preserve">Fees and contingency on works</t>
@@ -120,13 +120,13 @@
     <t xml:space="preserve">All England Club</t>
   </si>
   <si>
-    <t xml:space="preserve">New rent from 2028</t>
+    <t xml:space="preserve">New rent from completion</t>
   </si>
   <si>
     <t xml:space="preserve">£ pa</t>
   </si>
   <si>
-    <t xml:space="preserve">Current £350,000 received in 2027</t>
+    <t xml:space="preserve">All England Club rent from completion; surrender and regrant complete on the day of purchase</t>
   </si>
   <si>
     <t xml:space="preserve">Surrender premium to the Club</t>
@@ -138,30 +138,18 @@
     <t xml:space="preserve">Other lots</t>
   </si>
   <si>
-    <t xml:space="preserve">Cottages and Lodge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value of 1 and 2 Bank Lane and Clarence Lodge with vacant possession</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year the cottages are sold</t>
+    <t xml:space="preserve">National Tennis Centre reversion at exit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peppercorn to 2129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year the residential value is taken in</t>
   </si>
   <si>
     <t xml:space="preserve">year</t>
   </si>
   <si>
-    <t xml:space="preserve">0 = on completion; otherwise end of that year. Everything is sold at once at the end of the hold.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Tennis Centre reversion at exit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peppercorn to 2129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Year the Grange value is taken in</t>
-  </si>
-  <si>
     <t xml:space="preserve">Year the Grange value is taken in: 0 = on completion; otherwise end of that year. Everything is sold at once at the end of the hold.</t>
   </si>
   <si>
@@ -171,10 +159,10 @@
     <t xml:space="preserve">Grange holding cost until sold: 0 while Related's underwrite carries the conversion costs and value; c. £1,000,000 pa if held empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Grange value, placeholder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder value for The Grange pending Related's residential underwrite (Woody Bruce, 17 October 2026)</t>
+    <t xml:space="preserve">The Grange and cottages, placeholder value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder value for The Grange and the cottages together, pending Related's residential underwrite (Woody Bruce, 17 October 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Debt</t>
@@ -228,9 +216,6 @@
     <t xml:space="preserve">Grange price, £</t>
   </si>
   <si>
-    <t xml:space="preserve">Cottages, £</t>
-  </si>
-  <si>
     <t xml:space="preserve">NTC reversion, £</t>
   </si>
   <si>
@@ -249,7 +234,7 @@
     <t xml:space="preserve">Annual cash flow, £</t>
   </si>
   <si>
-    <t xml:space="preserve">Completion January 2027 (year 0). Third Space lease from January 2028 (year 2); capital contribution paid in year 2; Club surrender and £100,000 lease from 2028; exit at the end of the hold year. Rows beyond the hold year are zero.</t>
+    <t xml:space="preserve">Completion January 2027 (year 0): purchase, Third Space lease, capital contribution and the Club's surrender and regrant all on the same day. Nothing more spent on the leisure side; everything sold as one lot at the end of the hold year. Rows beyond the hold year are zero.</t>
   </si>
   <si>
     <t xml:space="preserve">Year</t>
@@ -318,7 +303,7 @@
     <t xml:space="preserve">Outputs</t>
   </si>
   <si>
-    <t xml:space="preserve">All figures recompute from Inputs. For the breakeven bid, Goal Seek Outputs!B13 to the target by changing Inputs!B5; for the Grange breakeven, change Inputs!B28 instead.</t>
+    <t xml:space="preserve">All figures recompute from Inputs. For the breakeven bid, Goal Seek Outputs!B13 to the target by changing the purchase price on Inputs; for the residential breakeven, change the Grange and cottages placeholder instead.</t>
   </si>
   <si>
     <t xml:space="preserve">Receipts</t>
@@ -327,12 +312,6 @@
     <t xml:space="preserve">Rent received during the hold</t>
   </si>
   <si>
-    <t xml:space="preserve">Cottages and Lodge, at sale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Grange, placeholder value</t>
-  </si>
-  <si>
     <t xml:space="preserve">Exit: Third Space, grounds and NTC reversion</t>
   </si>
   <si>
@@ -351,7 +330,7 @@
     <t xml:space="preserve">Total cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Profit on cost (B13 = profit / total cost)</t>
+    <t xml:space="preserve">Profit on cost</t>
   </si>
   <si>
     <t xml:space="preserve">Returns</t>
@@ -363,7 +342,7 @@
     <t xml:space="preserve">Profit on receipts</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield on cost, stabilised rent over cost net of Grange and cottages</t>
+    <t xml:space="preserve">Yield on cost, stabilised rent over cost net of the residential placeholder</t>
   </si>
   <si>
     <t xml:space="preserve">Unlevered IRR</t>
@@ -390,7 +369,7 @@
     <t xml:space="preserve">Let value: day-one rents at the exit yields, net of purchaser's costs, plus NTC reversion</t>
   </si>
   <si>
-    <t xml:space="preserve">Acquisition debt outstanding at letting (end of year 2)</t>
+    <t xml:space="preserve">Acquisition debt outstanding at letting (completion)</t>
   </si>
   <si>
     <t xml:space="preserve">Refinance loan</t>
@@ -872,7 +851,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1042,7 +1021,7 @@
         <v>25</v>
       </c>
       <c r="B15" s="8" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>26</v>
@@ -1136,7 +1115,7 @@
         <v>38</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>4</v>
@@ -1163,11 +1142,11 @@
       <c r="A25" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="9" t="n">
-        <v>0.5</v>
+      <c r="B25" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>44</v>
@@ -1177,272 +1156,233 @@
       <c r="A26" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="8" t="n">
-        <v>3</v>
+      <c r="B26" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>48</v>
-      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="6" t="n">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
       <c r="D29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="7" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>53</v>
-      </c>
+      <c r="D30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B31" s="7" t="n">
-        <v>0.07</v>
+        <v>0.55</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="2"/>
+      <c r="D31" s="3" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B32" s="7" t="n">
-        <v>0.015</v>
+        <v>0.06</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="7" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
+      <c r="B35" s="10" t="n">
+        <f aca="false">Inputs!$B$10*Inputs!$B$11</f>
+        <v>1804260</v>
+      </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B36" s="2"/>
+      <c r="A36" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="10" t="n">
+        <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
+        <v>0</v>
+      </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B37" s="10" t="n">
-        <f aca="false">Inputs!$B$10*Inputs!$B$11</f>
-        <v>1804260</v>
+        <f aca="false">B36*Inputs!$B$16</f>
+        <v>0</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B38" s="10" t="n">
-        <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
-        <v>4510650</v>
+        <f aca="false">B35*Inputs!$B$13</f>
+        <v>1804260</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B39" s="10" t="n">
-        <f aca="false">B38*Inputs!$B$16</f>
-        <v>676597.5</v>
+        <f aca="false">B35*Inputs!$B$12</f>
+        <v>3608520</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B40" s="10" t="n">
-        <f aca="false">B37*Inputs!$B$13</f>
-        <v>1804260</v>
+        <f aca="false">Inputs!$B$5*1000000</f>
+        <v>30000000</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B41" s="10" t="n">
-        <f aca="false">B37*Inputs!$B$12</f>
-        <v>3608520</v>
+        <f aca="false">Inputs!$B$26*1000000</f>
+        <v>7000000</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B42" s="10" t="n">
-        <f aca="false">Inputs!$B$5*1000000</f>
-        <v>30000000</v>
+        <f aca="false">Inputs!$B$23*1000000</f>
+        <v>500000</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B43" s="10" t="n">
-        <f aca="false">Inputs!$B$28*1000000</f>
-        <v>7000000</v>
+        <f aca="false">B35*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
+        <v>1804260</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B44" s="10" t="n">
-        <f aca="false">Inputs!$B$23*1000000</f>
-        <v>3000000</v>
+        <v>66</v>
+      </c>
+      <c r="B44" s="11" t="n">
+        <f aca="false">MAX(0,Inputs!$B$12-Inputs!$B$7)</f>
+        <v>0</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B45" s="10" t="n">
-        <f aca="false">Inputs!$B$25*1000000</f>
-        <v>500000</v>
+        <f aca="false">B43/Inputs!$B$17/(1+Inputs!$B$6)-B44*B43</f>
+        <v>22525093.6329588</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B46" s="10" t="n">
-        <f aca="false">B37*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
-        <v>1804260</v>
+        <f aca="false">Inputs!$B$19/Inputs!$B$21/(1+Inputs!$B$6)</f>
+        <v>1337613.69716426</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B47" s="11" t="n">
-        <f aca="false">MAX(0,Inputs!$B$12-(Inputs!$B$7-1))</f>
-        <v>0</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B48" s="10" t="n">
-        <f aca="false">B46/Inputs!$B$17/(1+Inputs!$B$6)-B47*B46</f>
-        <v>22525093.6329588</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B49" s="10" t="n">
-        <f aca="false">Inputs!$B$19/Inputs!$B$21/(1+Inputs!$B$6)</f>
-        <v>1337613.69716426</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1470,7 +1410,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1494,7 +1434,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1540,64 +1480,64 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="G4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="I4" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="L4" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="N4" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="O4" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="P4" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="Q4" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="R4" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="S4" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="T4" s="12" t="s">
         <v>90</v>
-      </c>
-      <c r="P4" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q4" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="R4" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="S4" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="T4" s="12" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,52 +1553,52 @@
         <v>1</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">C5*IF(A5=0,0,IF(A5=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C5*IF(A5=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">C5*IF(A5&lt;2,0,IF(A5-1&lt;=Inputs!$B$12,0,IF(A5-2&lt;Inputs!$B$12,A5-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A5-2)/5))))</f>
+        <f aca="false">C5*IF(A5&lt;1,0,IF(A5&lt;=Inputs!$B$12,0,IF(A5-1&lt;Inputs!$B$12,A5-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A5-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A5=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A5=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A5=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <f aca="false">-C5*(IF(A5=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A5=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A5=2,Inputs!$B$40,0))</f>
-        <v>-32040000</v>
+        <f aca="false">-C5*(IF(A5=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <v>-33844260</v>
       </c>
       <c r="H5" s="10" t="n">
-        <f aca="false">-C5*IF(AND(Inputs!$B$26&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C5*IF(AND(Inputs!$B$24&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I5" s="10" t="n">
-        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">SUM(D5:I5)</f>
-        <v>-32040000</v>
+        <v>-33844260</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">-G5-F5</f>
-        <v>32040000</v>
+        <v>33844260</v>
       </c>
       <c r="L5" s="10" t="n">
-        <f aca="false">IF(K5&gt;0,Inputs!$B$30*K5,0)</f>
-        <v>17622000</v>
+        <f aca="false">IF(K5&gt;0,Inputs!$B$28*K5,0)</f>
+        <v>18614343</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="N5" s="10" t="n">
-        <f aca="false">M5*Inputs!$B$31</f>
+        <f aca="false">M5*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O5" s="10" t="n">
-        <f aca="false">L5*Inputs!$B$32</f>
-        <v>264330</v>
+        <f aca="false">L5*Inputs!$B$30</f>
+        <v>279215.145</v>
       </c>
       <c r="P5" s="10" t="n">
         <f aca="false">IF(K5&lt;0,MIN(M5+L5,-K5),0)+IF(A5=Inputs!$B$7,M5+L5-IF(K5&lt;0,MIN(M5+L5,-K5),0),0)</f>
@@ -1666,19 +1606,19 @@
       </c>
       <c r="Q5" s="10" t="n">
         <f aca="false">M5+L5-P5</f>
-        <v>17622000</v>
+        <v>18614343</v>
       </c>
       <c r="R5" s="10" t="n">
         <f aca="false">L5-N5-P5-O5</f>
-        <v>17357670</v>
+        <v>18335127.855</v>
       </c>
       <c r="S5" s="10" t="n">
         <f aca="false">J5+R5</f>
-        <v>-14682330</v>
+        <v>-15509132.145</v>
       </c>
       <c r="T5" s="10" t="n">
         <f aca="false">S5</f>
-        <v>-14682330</v>
+        <v>-15509132.145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1694,52 +1634,52 @@
         <v>1</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">C6*IF(A6=0,0,IF(A6=1,350000,Inputs!$B$19))</f>
-        <v>350000</v>
+        <f aca="false">C6*IF(A6=0,0,Inputs!$B$19)</f>
+        <v>100000</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">C6*IF(A6&lt;2,0,IF(A6-1&lt;=Inputs!$B$12,0,IF(A6-2&lt;Inputs!$B$12,A6-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A6-2)/5))))</f>
+        <f aca="false">C6*IF(A6&lt;1,0,IF(A6&lt;=Inputs!$B$12,0,IF(A6-1&lt;Inputs!$B$12,A6-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A6-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A6=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A6=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A6=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">-C6*(IF(A6=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A6=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A6=2,Inputs!$B$40,0))</f>
-        <v>-5187247.5</v>
+        <f aca="false">-C6*(IF(A6=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A6=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <v>-0</v>
       </c>
       <c r="H6" s="10" t="n">
-        <f aca="false">-C6*IF(AND(Inputs!$B$26&gt;0,A6&gt;=1,A6&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C6*IF(AND(Inputs!$B$24&gt;0,A6&gt;=1,A6&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="10" t="n">
         <f aca="false">SUM(D6:I6)</f>
-        <v>-4837247.5</v>
+        <v>100000</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">-G6-F6</f>
-        <v>5187247.5</v>
+        <v>0</v>
       </c>
       <c r="L6" s="10" t="n">
-        <f aca="false">IF(K6&gt;0,Inputs!$B$30*K6,0)</f>
-        <v>2852986.125</v>
+        <f aca="false">IF(K6&gt;0,Inputs!$B$28*K6,0)</f>
+        <v>0</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">Q5</f>
-        <v>17622000</v>
+        <v>18614343</v>
       </c>
       <c r="N6" s="10" t="n">
-        <f aca="false">M6*Inputs!$B$31</f>
-        <v>1233540</v>
+        <f aca="false">M6*Inputs!$B$29</f>
+        <v>1303004.01</v>
       </c>
       <c r="O6" s="10" t="n">
-        <f aca="false">L6*Inputs!$B$32</f>
-        <v>42794.791875</v>
+        <f aca="false">L6*Inputs!$B$30</f>
+        <v>0</v>
       </c>
       <c r="P6" s="10" t="n">
         <f aca="false">IF(K6&lt;0,MIN(M6+L6,-K6),0)+IF(A6=Inputs!$B$7,M6+L6-IF(K6&lt;0,MIN(M6+L6,-K6),0),0)</f>
@@ -1747,19 +1687,19 @@
       </c>
       <c r="Q6" s="10" t="n">
         <f aca="false">M6+L6-P6</f>
-        <v>20474986.125</v>
+        <v>18614343</v>
       </c>
       <c r="R6" s="10" t="n">
         <f aca="false">L6-N6-P6-O6</f>
-        <v>1576651.333125</v>
+        <v>-1303004.01</v>
       </c>
       <c r="S6" s="10" t="n">
         <f aca="false">J6+R6</f>
-        <v>-3260596.166875</v>
+        <v>-1203004.01</v>
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">T5+S6</f>
-        <v>-17942926.166875</v>
+        <v>-16712136.155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1775,52 +1715,52 @@
         <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">C7*IF(A7=0,0,IF(A7=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C7*IF(A7=0,0,Inputs!$B$19)</f>
         <v>100000</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">C7*IF(A7&lt;2,0,IF(A7-1&lt;=Inputs!$B$12,0,IF(A7-2&lt;Inputs!$B$12,A7-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A7-2)/5))))</f>
+        <f aca="false">C7*IF(A7&lt;1,0,IF(A7&lt;=Inputs!$B$12,0,IF(A7-1&lt;Inputs!$B$12,A7-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A7-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A7=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A7=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A7=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
-        <f aca="false">-C7*(IF(A7=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A7=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A7=2,Inputs!$B$40,0))</f>
-        <v>-1804260</v>
+        <f aca="false">-C7*(IF(A7=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A7=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <v>-0</v>
       </c>
       <c r="H7" s="10" t="n">
-        <f aca="false">-C7*IF(AND(Inputs!$B$26&gt;0,A7&gt;=1,A7&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C7*IF(AND(Inputs!$B$24&gt;0,A7&gt;=1,A7&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I7" s="10" t="n">
-        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="10" t="n">
         <f aca="false">SUM(D7:I7)</f>
-        <v>-1704260</v>
+        <v>100000</v>
       </c>
       <c r="K7" s="10" t="n">
         <f aca="false">-G7-F7</f>
-        <v>1804260</v>
+        <v>0</v>
       </c>
       <c r="L7" s="10" t="n">
-        <f aca="false">IF(K7&gt;0,Inputs!$B$30*K7,0)</f>
-        <v>992343</v>
+        <f aca="false">IF(K7&gt;0,Inputs!$B$28*K7,0)</f>
+        <v>0</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">Q6</f>
-        <v>20474986.125</v>
+        <v>18614343</v>
       </c>
       <c r="N7" s="10" t="n">
-        <f aca="false">M7*Inputs!$B$31</f>
-        <v>1433249.02875</v>
+        <f aca="false">M7*Inputs!$B$29</f>
+        <v>1303004.01</v>
       </c>
       <c r="O7" s="10" t="n">
-        <f aca="false">L7*Inputs!$B$32</f>
-        <v>14885.145</v>
+        <f aca="false">L7*Inputs!$B$30</f>
+        <v>0</v>
       </c>
       <c r="P7" s="10" t="n">
         <f aca="false">IF(K7&lt;0,MIN(M7+L7,-K7),0)+IF(A7=Inputs!$B$7,M7+L7-IF(K7&lt;0,MIN(M7+L7,-K7),0),0)</f>
@@ -1828,19 +1768,19 @@
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">M7+L7-P7</f>
-        <v>21467329.125</v>
+        <v>18614343</v>
       </c>
       <c r="R7" s="10" t="n">
         <f aca="false">L7-N7-P7-O7</f>
-        <v>-455791.17375</v>
+        <v>-1303004.01</v>
       </c>
       <c r="S7" s="10" t="n">
         <f aca="false">J7+R7</f>
-        <v>-2160051.17375</v>
+        <v>-1203004.01</v>
       </c>
       <c r="T7" s="10" t="n">
         <f aca="false">T6+S7</f>
-        <v>-20102977.340625</v>
+        <v>-17915140.165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,56 +1796,56 @@
         <v>1</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">C8*IF(A8=0,0,IF(A8=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C8*IF(A8=0,0,Inputs!$B$19)</f>
         <v>100000</v>
       </c>
       <c r="E8" s="10" t="n">
-        <f aca="false">C8*IF(A8&lt;2,0,IF(A8-1&lt;=Inputs!$B$12,0,IF(A8-2&lt;Inputs!$B$12,A8-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A8-2)/5))))</f>
-        <v>0</v>
+        <f aca="false">C8*IF(A8&lt;1,0,IF(A8&lt;=Inputs!$B$12,0,IF(A8-1&lt;Inputs!$B$12,A8-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A8-1)/5))))</f>
+        <v>1804260</v>
       </c>
       <c r="F8" s="10" t="n">
-        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A8=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A8=Inputs!$B$26),Inputs!$B$43,0))</f>
-        <v>10000000</v>
+        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A8=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <v>7000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <f aca="false">-C8*(IF(A8=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A8=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A8=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C8*(IF(A8=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A8=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H8" s="10" t="n">
-        <f aca="false">-C8*IF(AND(Inputs!$B$26&gt;0,A8&gt;=1,A8&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C8*IF(AND(Inputs!$B$24&gt;0,A8&gt;=1,A8&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>24362707.3301231</v>
       </c>
       <c r="J8" s="10" t="n">
         <f aca="false">SUM(D8:I8)</f>
-        <v>34462707.3301231</v>
+        <v>33266967.3301231</v>
       </c>
       <c r="K8" s="10" t="n">
         <f aca="false">-G8-F8</f>
-        <v>-10000000</v>
+        <v>-7000000</v>
       </c>
       <c r="L8" s="10" t="n">
-        <f aca="false">IF(K8&gt;0,Inputs!$B$30*K8,0)</f>
+        <f aca="false">IF(K8&gt;0,Inputs!$B$28*K8,0)</f>
         <v>0</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">Q7</f>
-        <v>21467329.125</v>
+        <v>18614343</v>
       </c>
       <c r="N8" s="10" t="n">
-        <f aca="false">M8*Inputs!$B$31</f>
-        <v>1502713.03875</v>
+        <f aca="false">M8*Inputs!$B$29</f>
+        <v>1303004.01</v>
       </c>
       <c r="O8" s="10" t="n">
-        <f aca="false">L8*Inputs!$B$32</f>
+        <f aca="false">L8*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P8" s="10" t="n">
         <f aca="false">IF(K8&lt;0,MIN(M8+L8,-K8),0)+IF(A8=Inputs!$B$7,M8+L8-IF(K8&lt;0,MIN(M8+L8,-K8),0),0)</f>
-        <v>21467329.125</v>
+        <v>18614343</v>
       </c>
       <c r="Q8" s="10" t="n">
         <f aca="false">M8+L8-P8</f>
@@ -1913,15 +1853,15 @@
       </c>
       <c r="R8" s="10" t="n">
         <f aca="false">L8-N8-P8-O8</f>
-        <v>-22970042.16375</v>
+        <v>-19917347.01</v>
       </c>
       <c r="S8" s="10" t="n">
         <f aca="false">J8+R8</f>
-        <v>11492665.1663731</v>
+        <v>13349620.3201231</v>
       </c>
       <c r="T8" s="10" t="n">
         <f aca="false">T7+S8</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1937,27 +1877,27 @@
         <v>0</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">C9*IF(A9=0,0,IF(A9=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C9*IF(A9=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <f aca="false">C9*IF(A9&lt;2,0,IF(A9-1&lt;=Inputs!$B$12,0,IF(A9-2&lt;Inputs!$B$12,A9-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A9-2)/5))))</f>
+        <f aca="false">C9*IF(A9&lt;1,0,IF(A9&lt;=Inputs!$B$12,0,IF(A9-1&lt;Inputs!$B$12,A9-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A9-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
-        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A9=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A9=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A9=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
-        <f aca="false">-C9*(IF(A9=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A9=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A9=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C9*(IF(A9=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A9=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H9" s="10" t="n">
-        <f aca="false">-C9*IF(AND(Inputs!$B$26&gt;0,A9&gt;=1,A9&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C9*IF(AND(Inputs!$B$24&gt;0,A9&gt;=1,A9&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I9" s="10" t="n">
-        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="10" t="n">
@@ -1969,7 +1909,7 @@
         <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <f aca="false">IF(K9&gt;0,Inputs!$B$30*K9,0)</f>
+        <f aca="false">IF(K9&gt;0,Inputs!$B$28*K9,0)</f>
         <v>0</v>
       </c>
       <c r="M9" s="10" t="n">
@@ -1977,11 +1917,11 @@
         <v>0</v>
       </c>
       <c r="N9" s="10" t="n">
-        <f aca="false">M9*Inputs!$B$31</f>
+        <f aca="false">M9*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O9" s="10" t="n">
-        <f aca="false">L9*Inputs!$B$32</f>
+        <f aca="false">L9*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P9" s="10" t="n">
@@ -2002,7 +1942,7 @@
       </c>
       <c r="T9" s="10" t="n">
         <f aca="false">T8+S9</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2018,27 +1958,27 @@
         <v>0</v>
       </c>
       <c r="D10" s="10" t="n">
-        <f aca="false">C10*IF(A10=0,0,IF(A10=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C10*IF(A10=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <f aca="false">C10*IF(A10&lt;2,0,IF(A10-1&lt;=Inputs!$B$12,0,IF(A10-2&lt;Inputs!$B$12,A10-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A10-2)/5))))</f>
+        <f aca="false">C10*IF(A10&lt;1,0,IF(A10&lt;=Inputs!$B$12,0,IF(A10-1&lt;Inputs!$B$12,A10-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A10-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A10=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A10=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A10=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <f aca="false">-C10*(IF(A10=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A10=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A10=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C10*(IF(A10=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A10=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H10" s="10" t="n">
-        <f aca="false">-C10*IF(AND(Inputs!$B$26&gt;0,A10&gt;=1,A10&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C10*IF(AND(Inputs!$B$24&gt;0,A10&gt;=1,A10&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J10" s="10" t="n">
@@ -2050,7 +1990,7 @@
         <v>0</v>
       </c>
       <c r="L10" s="10" t="n">
-        <f aca="false">IF(K10&gt;0,Inputs!$B$30*K10,0)</f>
+        <f aca="false">IF(K10&gt;0,Inputs!$B$28*K10,0)</f>
         <v>0</v>
       </c>
       <c r="M10" s="10" t="n">
@@ -2058,11 +1998,11 @@
         <v>0</v>
       </c>
       <c r="N10" s="10" t="n">
-        <f aca="false">M10*Inputs!$B$31</f>
+        <f aca="false">M10*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O10" s="10" t="n">
-        <f aca="false">L10*Inputs!$B$32</f>
+        <f aca="false">L10*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P10" s="10" t="n">
@@ -2083,7 +2023,7 @@
       </c>
       <c r="T10" s="10" t="n">
         <f aca="false">T9+S10</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2099,27 +2039,27 @@
         <v>0</v>
       </c>
       <c r="D11" s="10" t="n">
-        <f aca="false">C11*IF(A11=0,0,IF(A11=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C11*IF(A11=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E11" s="10" t="n">
-        <f aca="false">C11*IF(A11&lt;2,0,IF(A11-1&lt;=Inputs!$B$12,0,IF(A11-2&lt;Inputs!$B$12,A11-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A11-2)/5))))</f>
+        <f aca="false">C11*IF(A11&lt;1,0,IF(A11&lt;=Inputs!$B$12,0,IF(A11-1&lt;Inputs!$B$12,A11-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A11-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F11" s="10" t="n">
-        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A11=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A11=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A11=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <f aca="false">-C11*(IF(A11=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A11=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A11=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C11*(IF(A11=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A11=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H11" s="10" t="n">
-        <f aca="false">-C11*IF(AND(Inputs!$B$26&gt;0,A11&gt;=1,A11&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C11*IF(AND(Inputs!$B$24&gt;0,A11&gt;=1,A11&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="10" t="n">
@@ -2131,7 +2071,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
-        <f aca="false">IF(K11&gt;0,Inputs!$B$30*K11,0)</f>
+        <f aca="false">IF(K11&gt;0,Inputs!$B$28*K11,0)</f>
         <v>0</v>
       </c>
       <c r="M11" s="10" t="n">
@@ -2139,11 +2079,11 @@
         <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
-        <f aca="false">M11*Inputs!$B$31</f>
+        <f aca="false">M11*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O11" s="10" t="n">
-        <f aca="false">L11*Inputs!$B$32</f>
+        <f aca="false">L11*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P11" s="10" t="n">
@@ -2164,7 +2104,7 @@
       </c>
       <c r="T11" s="10" t="n">
         <f aca="false">T10+S11</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2180,27 +2120,27 @@
         <v>0</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">C12*IF(A12=0,0,IF(A12=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C12*IF(A12=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <f aca="false">C12*IF(A12&lt;2,0,IF(A12-1&lt;=Inputs!$B$12,0,IF(A12-2&lt;Inputs!$B$12,A12-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A12-2)/5))))</f>
+        <f aca="false">C12*IF(A12&lt;1,0,IF(A12&lt;=Inputs!$B$12,0,IF(A12-1&lt;Inputs!$B$12,A12-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A12-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A12=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A12=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A12=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
-        <f aca="false">-C12*(IF(A12=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A12=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A12=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C12*(IF(A12=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A12=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H12" s="10" t="n">
-        <f aca="false">-C12*IF(AND(Inputs!$B$26&gt;0,A12&gt;=1,A12&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C12*IF(AND(Inputs!$B$24&gt;0,A12&gt;=1,A12&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J12" s="10" t="n">
@@ -2212,7 +2152,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="10" t="n">
-        <f aca="false">IF(K12&gt;0,Inputs!$B$30*K12,0)</f>
+        <f aca="false">IF(K12&gt;0,Inputs!$B$28*K12,0)</f>
         <v>0</v>
       </c>
       <c r="M12" s="10" t="n">
@@ -2220,11 +2160,11 @@
         <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
-        <f aca="false">M12*Inputs!$B$31</f>
+        <f aca="false">M12*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O12" s="10" t="n">
-        <f aca="false">L12*Inputs!$B$32</f>
+        <f aca="false">L12*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P12" s="10" t="n">
@@ -2245,7 +2185,7 @@
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">T11+S12</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2261,27 +2201,27 @@
         <v>0</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">C13*IF(A13=0,0,IF(A13=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C13*IF(A13=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">C13*IF(A13&lt;2,0,IF(A13-1&lt;=Inputs!$B$12,0,IF(A13-2&lt;Inputs!$B$12,A13-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A13-2)/5))))</f>
+        <f aca="false">C13*IF(A13&lt;1,0,IF(A13&lt;=Inputs!$B$12,0,IF(A13-1&lt;Inputs!$B$12,A13-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A13-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A13=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A13=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A13=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
-        <f aca="false">-C13*(IF(A13=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A13=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A13=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C13*(IF(A13=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A13=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H13" s="10" t="n">
-        <f aca="false">-C13*IF(AND(Inputs!$B$26&gt;0,A13&gt;=1,A13&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C13*IF(AND(Inputs!$B$24&gt;0,A13&gt;=1,A13&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I13" s="10" t="n">
-        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="10" t="n">
@@ -2293,7 +2233,7 @@
         <v>0</v>
       </c>
       <c r="L13" s="10" t="n">
-        <f aca="false">IF(K13&gt;0,Inputs!$B$30*K13,0)</f>
+        <f aca="false">IF(K13&gt;0,Inputs!$B$28*K13,0)</f>
         <v>0</v>
       </c>
       <c r="M13" s="10" t="n">
@@ -2301,11 +2241,11 @@
         <v>0</v>
       </c>
       <c r="N13" s="10" t="n">
-        <f aca="false">M13*Inputs!$B$31</f>
+        <f aca="false">M13*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O13" s="10" t="n">
-        <f aca="false">L13*Inputs!$B$32</f>
+        <f aca="false">L13*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P13" s="10" t="n">
@@ -2326,7 +2266,7 @@
       </c>
       <c r="T13" s="10" t="n">
         <f aca="false">T12+S13</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2342,27 +2282,27 @@
         <v>0</v>
       </c>
       <c r="D14" s="10" t="n">
-        <f aca="false">C14*IF(A14=0,0,IF(A14=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C14*IF(A14=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E14" s="10" t="n">
-        <f aca="false">C14*IF(A14&lt;2,0,IF(A14-1&lt;=Inputs!$B$12,0,IF(A14-2&lt;Inputs!$B$12,A14-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A14-2)/5))))</f>
+        <f aca="false">C14*IF(A14&lt;1,0,IF(A14&lt;=Inputs!$B$12,0,IF(A14-1&lt;Inputs!$B$12,A14-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A14-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
-        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A14=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A14=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A14=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
-        <f aca="false">-C14*(IF(A14=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A14=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A14=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C14*(IF(A14=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A14=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H14" s="10" t="n">
-        <f aca="false">-C14*IF(AND(Inputs!$B$26&gt;0,A14&gt;=1,A14&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C14*IF(AND(Inputs!$B$24&gt;0,A14&gt;=1,A14&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J14" s="10" t="n">
@@ -2374,7 +2314,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="10" t="n">
-        <f aca="false">IF(K14&gt;0,Inputs!$B$30*K14,0)</f>
+        <f aca="false">IF(K14&gt;0,Inputs!$B$28*K14,0)</f>
         <v>0</v>
       </c>
       <c r="M14" s="10" t="n">
@@ -2382,11 +2322,11 @@
         <v>0</v>
       </c>
       <c r="N14" s="10" t="n">
-        <f aca="false">M14*Inputs!$B$31</f>
+        <f aca="false">M14*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O14" s="10" t="n">
-        <f aca="false">L14*Inputs!$B$32</f>
+        <f aca="false">L14*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P14" s="10" t="n">
@@ -2407,7 +2347,7 @@
       </c>
       <c r="T14" s="10" t="n">
         <f aca="false">T13+S14</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2423,27 +2363,27 @@
         <v>0</v>
       </c>
       <c r="D15" s="10" t="n">
-        <f aca="false">C15*IF(A15=0,0,IF(A15=1,350000,Inputs!$B$19))</f>
+        <f aca="false">C15*IF(A15=0,0,Inputs!$B$19)</f>
         <v>0</v>
       </c>
       <c r="E15" s="10" t="n">
-        <f aca="false">C15*IF(A15&lt;2,0,IF(A15-1&lt;=Inputs!$B$12,0,IF(A15-2&lt;Inputs!$B$12,A15-1-Inputs!$B$12,1)*Inputs!$B$37*(1+Inputs!$B$14)^(5*INT((A15-2)/5))))</f>
+        <f aca="false">C15*IF(A15&lt;1,0,IF(A15&lt;=Inputs!$B$12,0,IF(A15-1&lt;Inputs!$B$12,A15-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A15-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F15" s="10" t="n">
-        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$26=0,Inputs!$B$43,0),0)+IF(A15=Inputs!$B$24,Inputs!$B$44,0)+IF(AND(Inputs!$B$26&gt;0,A15=Inputs!$B$26),Inputs!$B$43,0))</f>
+        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A15=Inputs!$B$24),Inputs!$B$41,0))</f>
         <v>0</v>
       </c>
       <c r="G15" s="10" t="n">
-        <f aca="false">-C15*(IF(A15=0,Inputs!$B$42*(1+Inputs!$B$6),0)+IF(A15=1,Inputs!$B$38+Inputs!$B$39+Inputs!$B$20,0)+IF(A15=2,Inputs!$B$40,0))</f>
+        <f aca="false">-C15*(IF(A15=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A15=1,Inputs!$B$36+Inputs!$B$37,0))</f>
         <v>-0</v>
       </c>
       <c r="H15" s="10" t="n">
-        <f aca="false">-C15*IF(AND(Inputs!$B$26&gt;0,A15&gt;=1,A15&lt;=Inputs!$B$26),Inputs!$B$27,0)</f>
+        <f aca="false">-C15*IF(AND(Inputs!$B$24&gt;0,A15&gt;=1,A15&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
         <v>-0</v>
       </c>
       <c r="I15" s="10" t="n">
-        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$48+Inputs!$B$49+Inputs!$B$45,0)</f>
+        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
         <v>0</v>
       </c>
       <c r="J15" s="10" t="n">
@@ -2455,7 +2395,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="10" t="n">
-        <f aca="false">IF(K15&gt;0,Inputs!$B$30*K15,0)</f>
+        <f aca="false">IF(K15&gt;0,Inputs!$B$28*K15,0)</f>
         <v>0</v>
       </c>
       <c r="M15" s="10" t="n">
@@ -2463,11 +2403,11 @@
         <v>0</v>
       </c>
       <c r="N15" s="10" t="n">
-        <f aca="false">M15*Inputs!$B$31</f>
+        <f aca="false">M15*Inputs!$B$29</f>
         <v>0</v>
       </c>
       <c r="O15" s="10" t="n">
-        <f aca="false">L15*Inputs!$B$32</f>
+        <f aca="false">L15*Inputs!$B$30</f>
         <v>0</v>
       </c>
       <c r="P15" s="10" t="n">
@@ -2488,30 +2428,30 @@
       </c>
       <c r="T15" s="10" t="n">
         <f aca="false">T14+S15</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="13" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="14" t="n">
         <f aca="false">SUM(D5:D15)</f>
-        <v>550000</v>
+        <v>300000</v>
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">SUM(E5:E15)</f>
-        <v>0</v>
+        <v>1804260</v>
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">SUM(F5:F15)</f>
-        <v>10000000</v>
+        <v>7000000</v>
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">SUM(G5:G15)</f>
-        <v>-39031507.5</v>
+        <v>-33844260</v>
       </c>
       <c r="H16" s="14" t="n">
         <f aca="false">SUM(H5:H15)</f>
@@ -2523,43 +2463,43 @@
       </c>
       <c r="J16" s="14" t="n">
         <f aca="false">SUM(J5:J15)</f>
-        <v>-4118800.16987694</v>
+        <v>-377292.669876941</v>
       </c>
       <c r="K16" s="14" t="n">
         <f aca="false">SUM(K5:K15)</f>
-        <v>29031507.5</v>
+        <v>26844260</v>
       </c>
       <c r="L16" s="14" t="n">
         <f aca="false">SUM(L5:L15)</f>
-        <v>21467329.125</v>
+        <v>18614343</v>
       </c>
       <c r="M16" s="14" t="n">
         <f aca="false">SUM(M5:M15)</f>
-        <v>59564315.25</v>
+        <v>55843029</v>
       </c>
       <c r="N16" s="14" t="n">
         <f aca="false">SUM(N5:N15)</f>
-        <v>4169502.0675</v>
+        <v>3909012.03</v>
       </c>
       <c r="O16" s="14" t="n">
         <f aca="false">SUM(O5:O15)</f>
-        <v>322009.936875</v>
+        <v>279215.145</v>
       </c>
       <c r="P16" s="14" t="n">
         <f aca="false">SUM(P5:P15)</f>
-        <v>21467329.125</v>
+        <v>18614343</v>
       </c>
       <c r="Q16" s="14" t="n">
         <f aca="false">SUM(Q5:Q15)</f>
-        <v>59564315.25</v>
+        <v>55843029</v>
       </c>
       <c r="R16" s="14" t="n">
         <f aca="false">SUM(R5:R15)</f>
-        <v>-4491512.004375</v>
+        <v>-4188227.175</v>
       </c>
       <c r="S16" s="14" t="n">
         <f aca="false">SUM(S5:S15)</f>
-        <v>-8610312.17425194</v>
+        <v>-4565519.84487694</v>
       </c>
       <c r="T16" s="2"/>
     </row>
@@ -2579,7 +2519,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="78"/>
@@ -2588,13 +2528,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B2" s="2"/>
     </row>
@@ -2604,250 +2544,241 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">'Cash flow'!D16+'Cash flow'!E16</f>
-        <v>550000</v>
+        <v>2104260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">Inputs!$B$44</f>
-        <v>3000000</v>
+        <f aca="false">Inputs!$B$41</f>
+        <v>7000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">Inputs!$B$43</f>
-        <v>7000000</v>
+        <f aca="false">'Cash flow'!I16</f>
+        <v>24362707.3301231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B8" s="10" t="n">
-        <f aca="false">'Cash flow'!I16</f>
-        <v>24362707.3301231</v>
+        <f aca="false">B5+B6+B7</f>
+        <v>33466967.3301231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" s="10" t="n">
-        <f aca="false">SUM(B5:B8)</f>
-        <v>34912707.3301231</v>
-      </c>
+      <c r="A9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="2"/>
+      <c r="A10" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <f aca="false">-'Cash flow'!G16-'Cash flow'!H16</f>
+        <v>33844260</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">-'Cash flow'!G16-'Cash flow'!H16</f>
-        <v>39031507.5</v>
+        <f aca="false">'Cash flow'!N16+'Cash flow'!O16</f>
+        <v>4188227.175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">'Cash flow'!N16+'Cash flow'!O16</f>
-        <v>4491512.004375</v>
+        <f aca="false">B10+B11</f>
+        <v>38032487.175</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B13" s="10" t="n">
-        <f aca="false">B11+B12</f>
-        <v>43523019.504375</v>
+        <v>102</v>
+      </c>
+      <c r="B13" s="15" t="n">
+        <f aca="false">(B8-B12)/B12</f>
+        <v>-0.120042631549956</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B14" s="15" t="n">
-        <f aca="false">(B9-B13)/B13</f>
-        <v>-0.19783352056689</v>
-      </c>
+      <c r="A14" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B15" s="2"/>
+      <c r="A15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <f aca="false">B8-B12</f>
+        <v>-4565519.84487694</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="10" t="n">
-        <f aca="false">B9-B13</f>
-        <v>-8610312.17425194</v>
+        <v>105</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <f aca="false">B15/B8</f>
+        <v>-0.136418690102452</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B17" s="15" t="n">
-        <f aca="false">B16/B9</f>
-        <v>-0.246624018379201</v>
+        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/(B10-Inputs!$B$41)</f>
+        <v>0.07093732514884</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B18" s="15" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/(B11-Inputs!$B$43-Inputs!$B$44)</f>
-        <v>0.0655928735357611</v>
+        <f aca="false">IRR('Cash flow'!J5:J15,-0.05)</f>
+        <v>-0.00374098634422967</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B19" s="15" t="n">
-        <f aca="false">IRR('Cash flow'!J5:J15)</f>
-        <v>-0.0397824334770132</v>
+        <f aca="false">IRR('Cash flow'!S5:S15,-0.2)</f>
+        <v>-0.100333173821733</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B20" s="15" t="n">
-        <f aca="false">IRR('Cash flow'!S5:S15)</f>
-        <v>-0.195509552228641</v>
+        <v>109</v>
+      </c>
+      <c r="B20" s="16" t="n">
+        <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
+        <v>0.745158575214701</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B21" s="16" t="n">
-        <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
-        <v>0.571689704049368</v>
+        <v>110</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <f aca="false">-MIN('Cash flow'!T5:T15)</f>
+        <v>17915140.165</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B22" s="10" t="n">
-        <f aca="false">-MIN('Cash flow'!T5:T15)</f>
-        <v>20102977.340625</v>
+        <f aca="false">MAX('Cash flow'!Q5:Q15)</f>
+        <v>18614343</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="10" t="n">
-        <f aca="false">MAX('Cash flow'!Q5:Q15)</f>
-        <v>21467329.125</v>
+        <v>112</v>
+      </c>
+      <c r="B23" s="15" t="n">
+        <f aca="false">(Inputs!$B$35+Inputs!$B$19-B22*Inputs!$B$29)/B21</f>
+        <v>0.0335613332891833</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B24" s="15" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$19-B23*Inputs!$B$31)/B22</f>
-        <v>0.0199745020076472</v>
-      </c>
+      <c r="A24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B25" s="2"/>
+      <c r="A25" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="10" t="n">
+        <f aca="false">(Inputs!$B$35/Inputs!$B$17+Inputs!$B$19/Inputs!$B$21)/(1+Inputs!$B$6)+Inputs!$B$42</f>
+        <v>24362707.3301231</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B26" s="10" t="n">
-        <f aca="false">(Inputs!$B$37/Inputs!$B$17+Inputs!$B$19/Inputs!$B$21)/(1+Inputs!$B$6)+Inputs!$B$45</f>
-        <v>24362707.3301231</v>
+        <f aca="false">'Cash flow'!Q5</f>
+        <v>18614343</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B27" s="10" t="n">
-        <f aca="false">'Cash flow'!Q7</f>
-        <v>21467329.125</v>
+        <f aca="false">B25*Inputs!$B$31</f>
+        <v>13399489.0315677</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B28" s="10" t="n">
-        <f aca="false">B26*Inputs!$B$33</f>
-        <v>13399489.0315677</v>
+        <f aca="false">B27-B26</f>
+        <v>-5214853.96843232</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B29" s="10" t="n">
-        <f aca="false">B28-B27</f>
-        <v>-8067840.09343232</v>
+        <v>118</v>
+      </c>
+      <c r="B29" s="15" t="n">
+        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/B27</f>
+        <v>0.142114374325303</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B30" s="15" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/B28</f>
-        <v>0.142114374325303</v>
+        <v>119</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/(B27*Inputs!$B$32)</f>
+        <v>2.36857290542172</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B31" s="16" t="n">
-        <f aca="false">(Inputs!$B$37+Inputs!$B$19)/(B28*Inputs!$B$34)</f>
-        <v>2.36857290542172</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B32" s="10" t="n">
-        <f aca="false">MAX(0,(B28*Inputs!$B$34-Inputs!$B$19)*Inputs!$B$12)</f>
+        <v>120</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <f aca="false">MAX(0,(B27*Inputs!$B$32-Inputs!$B$19)*Inputs!$B$12)</f>
         <v>1407938.68378812</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Roehampton: one acquisition loan at 50% of the valuation after lettings, 9%, no refinance
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="121">
   <si>
     <t xml:space="preserve">Roehampton Sports Ground Estate — underwrite model</t>
   </si>
@@ -168,10 +168,10 @@
     <t xml:space="preserve">Debt</t>
   </si>
   <si>
-    <t xml:space="preserve">Loan to cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drawn against purchase, works and incentives</t>
+    <t xml:space="preserve">Loan to value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One loan on purchase, sized on the valuation after the lettings; no refinance</t>
   </si>
   <si>
     <t xml:space="preserve">All-in interest rate</t>
@@ -180,16 +180,7 @@
     <t xml:space="preserve">Arrangement and exit fees</t>
   </si>
   <si>
-    <t xml:space="preserve">% of draws</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refinance LTV once let</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investment loan against the let value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refinance all-in rate</t>
+    <t xml:space="preserve">% of the loan</t>
   </si>
   <si>
     <t xml:space="preserve">Derived</t>
@@ -231,6 +222,15 @@
     <t xml:space="preserve">Grounds value at exit, £</t>
   </si>
   <si>
+    <t xml:space="preserve">Valuation after the lettings, £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day-one cost, £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan drawn on completion, £</t>
+  </si>
+  <si>
     <t xml:space="preserve">Annual cash flow, £</t>
   </si>
   <si>
@@ -363,19 +363,19 @@
     <t xml:space="preserve">Cash on cash, first full rent year if held</t>
   </si>
   <si>
-    <t xml:space="preserve">Debt once the Third Space lease is signed and the Grange approved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Let value: day-one rents at the exit yields, net of purchaser's costs, plus NTC reversion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acquisition debt outstanding at letting (completion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refinance loan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equity released or (shortfall)</t>
+    <t xml:space="preserve">Debt on purchase, sized on the valuation after the lettings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuation after the lettings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan drawn on completion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan to cost, implied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity on day one</t>
   </si>
   <si>
     <t xml:space="preserve">Debt yield</t>
@@ -384,7 +384,7 @@
     <t xml:space="preserve">Interest cover once rent is paying</t>
   </si>
   <si>
-    <t xml:space="preserve">Interest reserve for the rent-free period</t>
+    <t xml:space="preserve">Interest shortfall during the rent-free</t>
   </si>
 </sst>
 </file>
@@ -851,7 +851,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1179,7 +1179,7 @@
         <v>48</v>
       </c>
       <c r="B28" s="7" t="n">
-        <v>0.55</v>
+        <v>0.5</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>7</v>
@@ -1193,7 +1193,7 @@
         <v>50</v>
       </c>
       <c r="B29" s="7" t="n">
-        <v>0.07</v>
+        <v>0.09</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>7</v>
@@ -1213,176 +1213,183 @@
       <c r="D30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="3" t="s">
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="B33" s="10" t="n">
+        <f aca="false">Inputs!$B$10*Inputs!$B$11</f>
+        <v>1804260</v>
+      </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="2"/>
+      <c r="A34" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
+        <v>0</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" s="10" t="n">
-        <f aca="false">Inputs!$B$10*Inputs!$B$11</f>
-        <v>1804260</v>
+        <f aca="false">B34*Inputs!$B$16</f>
+        <v>0</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="10" t="n">
-        <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
-        <v>0</v>
+        <f aca="false">B33*Inputs!$B$13</f>
+        <v>1804260</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" s="10" t="n">
-        <f aca="false">B36*Inputs!$B$16</f>
-        <v>0</v>
+        <f aca="false">B33*Inputs!$B$12</f>
+        <v>3608520</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" s="10" t="n">
-        <f aca="false">B35*Inputs!$B$13</f>
-        <v>1804260</v>
+        <f aca="false">Inputs!$B$5*1000000</f>
+        <v>30000000</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B39" s="10" t="n">
-        <f aca="false">B35*Inputs!$B$12</f>
-        <v>3608520</v>
+        <f aca="false">Inputs!$B$26*1000000</f>
+        <v>7000000</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B40" s="10" t="n">
-        <f aca="false">Inputs!$B$5*1000000</f>
-        <v>30000000</v>
+        <f aca="false">Inputs!$B$23*1000000</f>
+        <v>500000</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B41" s="10" t="n">
-        <f aca="false">Inputs!$B$26*1000000</f>
-        <v>7000000</v>
+        <f aca="false">B33*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
+        <v>1804260</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B42" s="10" t="n">
-        <f aca="false">Inputs!$B$23*1000000</f>
-        <v>500000</v>
+        <v>63</v>
+      </c>
+      <c r="B42" s="11" t="n">
+        <f aca="false">MAX(0,Inputs!$B$12-Inputs!$B$7)</f>
+        <v>0</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B43" s="10" t="n">
-        <f aca="false">B35*(1+Inputs!$B$14)^(5*INT((Inputs!$B$7-1)/5))</f>
-        <v>1804260</v>
+        <f aca="false">B41/Inputs!$B$17/(1+Inputs!$B$6)-B42*B41</f>
+        <v>22525093.6329588</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" s="11" t="n">
-        <f aca="false">MAX(0,Inputs!$B$12-Inputs!$B$7)</f>
-        <v>0</v>
+        <v>65</v>
+      </c>
+      <c r="B44" s="10" t="n">
+        <f aca="false">Inputs!$B$19/Inputs!$B$21/(1+Inputs!$B$6)</f>
+        <v>1337613.69716426</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45" s="10" t="n">
-        <f aca="false">B43/Inputs!$B$17/(1+Inputs!$B$6)-B44*B43</f>
-        <v>22525093.6329588</v>
+        <f aca="false">B33/Inputs!$B$17/(1+Inputs!$B$6)+B44+B40+B39</f>
+        <v>31362707.3301231</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B46" s="10" t="n">
-        <f aca="false">Inputs!$B$19/Inputs!$B$21/(1+Inputs!$B$6)</f>
-        <v>1337613.69716426</v>
+        <f aca="false">B38*(1+Inputs!$B$6)+B36+Inputs!$B$20</f>
+        <v>33844260</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47" s="10" t="n">
+        <f aca="false">MIN(Inputs!$B$28*B45,B46)</f>
+        <v>15681353.6650615</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1557,15 +1564,15 @@
         <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">C5*IF(A5&lt;1,0,IF(A5&lt;=Inputs!$B$12,0,IF(A5-1&lt;Inputs!$B$12,A5-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A5-1)/5))))</f>
+        <f aca="false">C5*IF(A5&lt;1,0,IF(A5&lt;=Inputs!$B$12,0,IF(A5-1&lt;Inputs!$B$12,A5-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A5-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A5=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C5*(IF(A5=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A5=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <f aca="false">-C5*(IF(A5=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C5*(IF(A5=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-33844260</v>
       </c>
       <c r="H5" s="10" t="n">
@@ -1573,7 +1580,7 @@
         <v>-0</v>
       </c>
       <c r="I5" s="10" t="n">
-        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A5=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J5" s="10" t="n">
@@ -1585,8 +1592,8 @@
         <v>33844260</v>
       </c>
       <c r="L5" s="10" t="n">
-        <f aca="false">IF(K5&gt;0,Inputs!$B$28*K5,0)</f>
-        <v>18614343</v>
+        <f aca="false">IF(A5=0,Inputs!$B$47,0)</f>
+        <v>15681353.6650615</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">0</f>
@@ -1598,7 +1605,7 @@
       </c>
       <c r="O5" s="10" t="n">
         <f aca="false">L5*Inputs!$B$30</f>
-        <v>279215.145</v>
+        <v>235220.304975923</v>
       </c>
       <c r="P5" s="10" t="n">
         <f aca="false">IF(K5&lt;0,MIN(M5+L5,-K5),0)+IF(A5=Inputs!$B$7,M5+L5-IF(K5&lt;0,MIN(M5+L5,-K5),0),0)</f>
@@ -1606,19 +1613,19 @@
       </c>
       <c r="Q5" s="10" t="n">
         <f aca="false">M5+L5-P5</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="R5" s="10" t="n">
         <f aca="false">L5-N5-P5-O5</f>
-        <v>18335127.855</v>
+        <v>15446133.3600856</v>
       </c>
       <c r="S5" s="10" t="n">
         <f aca="false">J5+R5</f>
-        <v>-15509132.145</v>
+        <v>-18398126.6399144</v>
       </c>
       <c r="T5" s="10" t="n">
         <f aca="false">S5</f>
-        <v>-15509132.145</v>
+        <v>-18398126.6399144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1638,15 +1645,15 @@
         <v>100000</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">C6*IF(A6&lt;1,0,IF(A6&lt;=Inputs!$B$12,0,IF(A6-1&lt;Inputs!$B$12,A6-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A6-1)/5))))</f>
+        <f aca="false">C6*IF(A6&lt;1,0,IF(A6&lt;=Inputs!$B$12,0,IF(A6-1&lt;Inputs!$B$12,A6-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A6-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A6=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C6*(IF(A6=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A6=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">-C6*(IF(A6=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A6=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C6*(IF(A6=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A6=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H6" s="10" t="n">
@@ -1654,7 +1661,7 @@
         <v>-0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A6=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J6" s="10" t="n">
@@ -1666,16 +1673,16 @@
         <v>0</v>
       </c>
       <c r="L6" s="10" t="n">
-        <f aca="false">IF(K6&gt;0,Inputs!$B$28*K6,0)</f>
+        <f aca="false">IF(A6=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M6" s="10" t="n">
         <f aca="false">Q5</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="N6" s="10" t="n">
         <f aca="false">M6*Inputs!$B$29</f>
-        <v>1303004.01</v>
+        <v>1411321.82985554</v>
       </c>
       <c r="O6" s="10" t="n">
         <f aca="false">L6*Inputs!$B$30</f>
@@ -1687,19 +1694,19 @@
       </c>
       <c r="Q6" s="10" t="n">
         <f aca="false">M6+L6-P6</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="R6" s="10" t="n">
         <f aca="false">L6-N6-P6-O6</f>
-        <v>-1303004.01</v>
+        <v>-1411321.82985554</v>
       </c>
       <c r="S6" s="10" t="n">
         <f aca="false">J6+R6</f>
-        <v>-1203004.01</v>
+        <v>-1311321.82985554</v>
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">T5+S6</f>
-        <v>-16712136.155</v>
+        <v>-19709448.4697699</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1719,15 +1726,15 @@
         <v>100000</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">C7*IF(A7&lt;1,0,IF(A7&lt;=Inputs!$B$12,0,IF(A7-1&lt;Inputs!$B$12,A7-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A7-1)/5))))</f>
+        <f aca="false">C7*IF(A7&lt;1,0,IF(A7&lt;=Inputs!$B$12,0,IF(A7-1&lt;Inputs!$B$12,A7-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A7-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A7=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A7=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
-        <f aca="false">-C7*(IF(A7=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A7=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C7*(IF(A7=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A7=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H7" s="10" t="n">
@@ -1735,7 +1742,7 @@
         <v>-0</v>
       </c>
       <c r="I7" s="10" t="n">
-        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A7=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J7" s="10" t="n">
@@ -1747,16 +1754,16 @@
         <v>0</v>
       </c>
       <c r="L7" s="10" t="n">
-        <f aca="false">IF(K7&gt;0,Inputs!$B$28*K7,0)</f>
+        <f aca="false">IF(A7=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M7" s="10" t="n">
         <f aca="false">Q6</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="N7" s="10" t="n">
         <f aca="false">M7*Inputs!$B$29</f>
-        <v>1303004.01</v>
+        <v>1411321.82985554</v>
       </c>
       <c r="O7" s="10" t="n">
         <f aca="false">L7*Inputs!$B$30</f>
@@ -1768,19 +1775,19 @@
       </c>
       <c r="Q7" s="10" t="n">
         <f aca="false">M7+L7-P7</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="R7" s="10" t="n">
         <f aca="false">L7-N7-P7-O7</f>
-        <v>-1303004.01</v>
+        <v>-1411321.82985554</v>
       </c>
       <c r="S7" s="10" t="n">
         <f aca="false">J7+R7</f>
-        <v>-1203004.01</v>
+        <v>-1311321.82985554</v>
       </c>
       <c r="T7" s="10" t="n">
         <f aca="false">T6+S7</f>
-        <v>-17915140.165</v>
+        <v>-21020770.2996255</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1800,15 +1807,15 @@
         <v>100000</v>
       </c>
       <c r="E8" s="10" t="n">
-        <f aca="false">C8*IF(A8&lt;1,0,IF(A8&lt;=Inputs!$B$12,0,IF(A8-1&lt;Inputs!$B$12,A8-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A8-1)/5))))</f>
+        <f aca="false">C8*IF(A8&lt;1,0,IF(A8&lt;=Inputs!$B$12,0,IF(A8-1&lt;Inputs!$B$12,A8-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A8-1)/5))))</f>
         <v>1804260</v>
       </c>
       <c r="F8" s="10" t="n">
-        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A8=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C8*(IF(A8=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A8=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>7000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <f aca="false">-C8*(IF(A8=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A8=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C8*(IF(A8=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A8=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H8" s="10" t="n">
@@ -1816,7 +1823,7 @@
         <v>-0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A8=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>24362707.3301231</v>
       </c>
       <c r="J8" s="10" t="n">
@@ -1828,16 +1835,16 @@
         <v>-7000000</v>
       </c>
       <c r="L8" s="10" t="n">
-        <f aca="false">IF(K8&gt;0,Inputs!$B$28*K8,0)</f>
+        <f aca="false">IF(A8=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">Q7</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="N8" s="10" t="n">
         <f aca="false">M8*Inputs!$B$29</f>
-        <v>1303004.01</v>
+        <v>1411321.82985554</v>
       </c>
       <c r="O8" s="10" t="n">
         <f aca="false">L8*Inputs!$B$30</f>
@@ -1845,7 +1852,7 @@
       </c>
       <c r="P8" s="10" t="n">
         <f aca="false">IF(K8&lt;0,MIN(M8+L8,-K8),0)+IF(A8=Inputs!$B$7,M8+L8-IF(K8&lt;0,MIN(M8+L8,-K8),0),0)</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="Q8" s="10" t="n">
         <f aca="false">M8+L8-P8</f>
@@ -1853,15 +1860,15 @@
       </c>
       <c r="R8" s="10" t="n">
         <f aca="false">L8-N8-P8-O8</f>
-        <v>-19917347.01</v>
+        <v>-17092675.4949171</v>
       </c>
       <c r="S8" s="10" t="n">
         <f aca="false">J8+R8</f>
-        <v>13349620.3201231</v>
+        <v>16174291.835206</v>
       </c>
       <c r="T8" s="10" t="n">
         <f aca="false">T7+S8</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,15 +1888,15 @@
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <f aca="false">C9*IF(A9&lt;1,0,IF(A9&lt;=Inputs!$B$12,0,IF(A9-1&lt;Inputs!$B$12,A9-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A9-1)/5))))</f>
+        <f aca="false">C9*IF(A9&lt;1,0,IF(A9&lt;=Inputs!$B$12,0,IF(A9-1&lt;Inputs!$B$12,A9-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A9-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
-        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A9=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C9*(IF(A9=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A9=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
-        <f aca="false">-C9*(IF(A9=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A9=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C9*(IF(A9=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A9=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H9" s="10" t="n">
@@ -1897,7 +1904,7 @@
         <v>-0</v>
       </c>
       <c r="I9" s="10" t="n">
-        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A9=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J9" s="10" t="n">
@@ -1909,7 +1916,7 @@
         <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <f aca="false">IF(K9&gt;0,Inputs!$B$28*K9,0)</f>
+        <f aca="false">IF(A9=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M9" s="10" t="n">
@@ -1942,7 +1949,7 @@
       </c>
       <c r="T9" s="10" t="n">
         <f aca="false">T8+S9</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1962,15 +1969,15 @@
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <f aca="false">C10*IF(A10&lt;1,0,IF(A10&lt;=Inputs!$B$12,0,IF(A10-1&lt;Inputs!$B$12,A10-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A10-1)/5))))</f>
+        <f aca="false">C10*IF(A10&lt;1,0,IF(A10&lt;=Inputs!$B$12,0,IF(A10-1&lt;Inputs!$B$12,A10-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A10-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A10=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C10*(IF(A10=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A10=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <f aca="false">-C10*(IF(A10=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A10=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C10*(IF(A10=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A10=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H10" s="10" t="n">
@@ -1978,7 +1985,7 @@
         <v>-0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A10=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J10" s="10" t="n">
@@ -1990,7 +1997,7 @@
         <v>0</v>
       </c>
       <c r="L10" s="10" t="n">
-        <f aca="false">IF(K10&gt;0,Inputs!$B$28*K10,0)</f>
+        <f aca="false">IF(A10=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M10" s="10" t="n">
@@ -2023,7 +2030,7 @@
       </c>
       <c r="T10" s="10" t="n">
         <f aca="false">T9+S10</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2043,15 +2050,15 @@
         <v>0</v>
       </c>
       <c r="E11" s="10" t="n">
-        <f aca="false">C11*IF(A11&lt;1,0,IF(A11&lt;=Inputs!$B$12,0,IF(A11-1&lt;Inputs!$B$12,A11-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A11-1)/5))))</f>
+        <f aca="false">C11*IF(A11&lt;1,0,IF(A11&lt;=Inputs!$B$12,0,IF(A11-1&lt;Inputs!$B$12,A11-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A11-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F11" s="10" t="n">
-        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A11=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C11*(IF(A11=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A11=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <f aca="false">-C11*(IF(A11=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A11=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C11*(IF(A11=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A11=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H11" s="10" t="n">
@@ -2059,7 +2066,7 @@
         <v>-0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A11=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J11" s="10" t="n">
@@ -2071,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
-        <f aca="false">IF(K11&gt;0,Inputs!$B$28*K11,0)</f>
+        <f aca="false">IF(A11=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M11" s="10" t="n">
@@ -2104,7 +2111,7 @@
       </c>
       <c r="T11" s="10" t="n">
         <f aca="false">T10+S11</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2124,15 +2131,15 @@
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <f aca="false">C12*IF(A12&lt;1,0,IF(A12&lt;=Inputs!$B$12,0,IF(A12-1&lt;Inputs!$B$12,A12-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A12-1)/5))))</f>
+        <f aca="false">C12*IF(A12&lt;1,0,IF(A12&lt;=Inputs!$B$12,0,IF(A12-1&lt;Inputs!$B$12,A12-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A12-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A12=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C12*(IF(A12=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A12=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
-        <f aca="false">-C12*(IF(A12=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A12=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C12*(IF(A12=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A12=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H12" s="10" t="n">
@@ -2140,7 +2147,7 @@
         <v>-0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A12=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J12" s="10" t="n">
@@ -2152,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="10" t="n">
-        <f aca="false">IF(K12&gt;0,Inputs!$B$28*K12,0)</f>
+        <f aca="false">IF(A12=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M12" s="10" t="n">
@@ -2185,7 +2192,7 @@
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">T11+S12</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2205,15 +2212,15 @@
         <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">C13*IF(A13&lt;1,0,IF(A13&lt;=Inputs!$B$12,0,IF(A13-1&lt;Inputs!$B$12,A13-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A13-1)/5))))</f>
+        <f aca="false">C13*IF(A13&lt;1,0,IF(A13&lt;=Inputs!$B$12,0,IF(A13-1&lt;Inputs!$B$12,A13-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A13-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A13=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C13*(IF(A13=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A13=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
-        <f aca="false">-C13*(IF(A13=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A13=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C13*(IF(A13=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A13=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H13" s="10" t="n">
@@ -2221,7 +2228,7 @@
         <v>-0</v>
       </c>
       <c r="I13" s="10" t="n">
-        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A13=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J13" s="10" t="n">
@@ -2233,7 +2240,7 @@
         <v>0</v>
       </c>
       <c r="L13" s="10" t="n">
-        <f aca="false">IF(K13&gt;0,Inputs!$B$28*K13,0)</f>
+        <f aca="false">IF(A13=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M13" s="10" t="n">
@@ -2266,7 +2273,7 @@
       </c>
       <c r="T13" s="10" t="n">
         <f aca="false">T12+S13</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2286,15 +2293,15 @@
         <v>0</v>
       </c>
       <c r="E14" s="10" t="n">
-        <f aca="false">C14*IF(A14&lt;1,0,IF(A14&lt;=Inputs!$B$12,0,IF(A14-1&lt;Inputs!$B$12,A14-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A14-1)/5))))</f>
+        <f aca="false">C14*IF(A14&lt;1,0,IF(A14&lt;=Inputs!$B$12,0,IF(A14-1&lt;Inputs!$B$12,A14-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A14-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
-        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A14=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C14*(IF(A14=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A14=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
-        <f aca="false">-C14*(IF(A14=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A14=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C14*(IF(A14=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A14=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H14" s="10" t="n">
@@ -2302,7 +2309,7 @@
         <v>-0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A14=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J14" s="10" t="n">
@@ -2314,7 +2321,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="10" t="n">
-        <f aca="false">IF(K14&gt;0,Inputs!$B$28*K14,0)</f>
+        <f aca="false">IF(A14=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M14" s="10" t="n">
@@ -2347,7 +2354,7 @@
       </c>
       <c r="T14" s="10" t="n">
         <f aca="false">T13+S14</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2367,15 +2374,15 @@
         <v>0</v>
       </c>
       <c r="E15" s="10" t="n">
-        <f aca="false">C15*IF(A15&lt;1,0,IF(A15&lt;=Inputs!$B$12,0,IF(A15-1&lt;Inputs!$B$12,A15-Inputs!$B$12,1)*Inputs!$B$35*(1+Inputs!$B$14)^(5*INT((A15-1)/5))))</f>
+        <f aca="false">C15*IF(A15&lt;1,0,IF(A15&lt;=Inputs!$B$12,0,IF(A15-1&lt;Inputs!$B$12,A15-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A15-1)/5))))</f>
         <v>0</v>
       </c>
       <c r="F15" s="10" t="n">
-        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$24=0,Inputs!$B$41,0),0)+IF(AND(Inputs!$B$24&gt;0,A15=Inputs!$B$24),Inputs!$B$41,0))</f>
+        <f aca="false">C15*(IF(A15=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A15=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G15" s="10" t="n">
-        <f aca="false">-C15*(IF(A15=0,Inputs!$B$40*(1+Inputs!$B$6)+Inputs!$B$38+Inputs!$B$20,0)+IF(A15=1,Inputs!$B$36+Inputs!$B$37,0))</f>
+        <f aca="false">-C15*(IF(A15=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A15=1,Inputs!$B$34+Inputs!$B$35,0))</f>
         <v>-0</v>
       </c>
       <c r="H15" s="10" t="n">
@@ -2383,7 +2390,7 @@
         <v>-0</v>
       </c>
       <c r="I15" s="10" t="n">
-        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$45+Inputs!$B$46+Inputs!$B$42,0)</f>
+        <f aca="false">IF(A15=Inputs!$B$7,Inputs!$B$43+Inputs!$B$44+Inputs!$B$40,0)</f>
         <v>0</v>
       </c>
       <c r="J15" s="10" t="n">
@@ -2395,7 +2402,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="10" t="n">
-        <f aca="false">IF(K15&gt;0,Inputs!$B$28*K15,0)</f>
+        <f aca="false">IF(A15=0,Inputs!$B$47,0)</f>
         <v>0</v>
       </c>
       <c r="M15" s="10" t="n">
@@ -2428,7 +2435,7 @@
       </c>
       <c r="T15" s="10" t="n">
         <f aca="false">T14+S15</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2471,35 +2478,35 @@
       </c>
       <c r="L16" s="14" t="n">
         <f aca="false">SUM(L5:L15)</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="M16" s="14" t="n">
         <f aca="false">SUM(M5:M15)</f>
-        <v>55843029</v>
+        <v>47044060.9951846</v>
       </c>
       <c r="N16" s="14" t="n">
         <f aca="false">SUM(N5:N15)</f>
-        <v>3909012.03</v>
+        <v>4233965.48956661</v>
       </c>
       <c r="O16" s="14" t="n">
         <f aca="false">SUM(O5:O15)</f>
-        <v>279215.145</v>
+        <v>235220.304975923</v>
       </c>
       <c r="P16" s="14" t="n">
         <f aca="false">SUM(P5:P15)</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
       <c r="Q16" s="14" t="n">
         <f aca="false">SUM(Q5:Q15)</f>
-        <v>55843029</v>
+        <v>47044060.9951846</v>
       </c>
       <c r="R16" s="14" t="n">
         <f aca="false">SUM(R5:R15)</f>
-        <v>-4188227.175</v>
+        <v>-4469185.79454254</v>
       </c>
       <c r="S16" s="14" t="n">
         <f aca="false">SUM(S5:S15)</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
       <c r="T16" s="2"/>
     </row>
@@ -2562,7 +2569,7 @@
         <v>45</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">Inputs!$B$41</f>
+        <f aca="false">Inputs!$B$39</f>
         <v>7000000</v>
       </c>
     </row>
@@ -2605,7 +2612,7 @@
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">'Cash flow'!N16+'Cash flow'!O16</f>
-        <v>4188227.175</v>
+        <v>4469185.79454254</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2614,7 +2621,7 @@
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">B10+B11</f>
-        <v>38032487.175</v>
+        <v>38313445.7945425</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2623,7 +2630,7 @@
       </c>
       <c r="B13" s="15" t="n">
         <f aca="false">(B8-B12)/B12</f>
-        <v>-0.120042631549956</v>
+        <v>-0.126495499527997</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2638,7 +2645,7 @@
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">B8-B12</f>
-        <v>-4565519.84487694</v>
+        <v>-4846478.46441948</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2647,7 +2654,7 @@
       </c>
       <c r="B16" s="15" t="n">
         <f aca="false">B15/B8</f>
-        <v>-0.136418690102452</v>
+        <v>-0.144813792555899</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2655,7 +2662,7 @@
         <v>106</v>
       </c>
       <c r="B17" s="15" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/(B10-Inputs!$B$41)</f>
+        <f aca="false">(Inputs!$B$33+Inputs!$B$19)/(B10-Inputs!$B$39)</f>
         <v>0.07093732514884</v>
       </c>
     </row>
@@ -2674,7 +2681,7 @@
       </c>
       <c r="B19" s="15" t="n">
         <f aca="false">IRR('Cash flow'!S5:S15,-0.2)</f>
-        <v>-0.100333173821733</v>
+        <v>-0.0893772076578962</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2683,7 +2690,7 @@
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
-        <v>0.745158575214701</v>
+        <v>0.769443346017352</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2692,7 +2699,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">-MIN('Cash flow'!T5:T15)</f>
-        <v>17915140.165</v>
+        <v>21020770.2996255</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2701,7 +2708,7 @@
       </c>
       <c r="B22" s="10" t="n">
         <f aca="false">MAX('Cash flow'!Q5:Q15)</f>
-        <v>18614343</v>
+        <v>15681353.6650615</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2709,8 +2716,8 @@
         <v>112</v>
       </c>
       <c r="B23" s="15" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$19-B22*Inputs!$B$29)/B21</f>
-        <v>0.0335613332891833</v>
+        <f aca="false">(Inputs!$B$33+Inputs!$B$19-B22*Inputs!$B$29)/B21</f>
+        <v>0.0234500526440387</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2724,8 +2731,8 @@
         <v>114</v>
       </c>
       <c r="B25" s="10" t="n">
-        <f aca="false">(Inputs!$B$35/Inputs!$B$17+Inputs!$B$19/Inputs!$B$21)/(1+Inputs!$B$6)+Inputs!$B$42</f>
-        <v>24362707.3301231</v>
+        <f aca="false">Inputs!$B$45</f>
+        <v>31362707.3301231</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2733,17 +2740,17 @@
         <v>115</v>
       </c>
       <c r="B26" s="10" t="n">
-        <f aca="false">'Cash flow'!Q5</f>
-        <v>18614343</v>
+        <f aca="false">Inputs!$B$47</f>
+        <v>15681353.6650615</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B27" s="10" t="n">
-        <f aca="false">B25*Inputs!$B$31</f>
-        <v>13399489.0315677</v>
+      <c r="B27" s="15" t="n">
+        <f aca="false">Inputs!$B$47/Inputs!$B$46</f>
+        <v>0.463338647825703</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2751,8 +2758,8 @@
         <v>117</v>
       </c>
       <c r="B28" s="10" t="n">
-        <f aca="false">B27-B26</f>
-        <v>-5214853.96843232</v>
+        <f aca="false">Inputs!$B$46-Inputs!$B$47</f>
+        <v>18162906.3349385</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2760,8 +2767,8 @@
         <v>118</v>
       </c>
       <c r="B29" s="15" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/B27</f>
-        <v>0.142114374325303</v>
+        <f aca="false">(Inputs!$B$33+Inputs!$B$19)/Inputs!$B$47</f>
+        <v>0.121434669523636</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2769,8 +2776,8 @@
         <v>119</v>
       </c>
       <c r="B30" s="16" t="n">
-        <f aca="false">(Inputs!$B$35+Inputs!$B$19)/(B27*Inputs!$B$32)</f>
-        <v>2.36857290542172</v>
+        <f aca="false">(Inputs!$B$33+Inputs!$B$19)/(Inputs!$B$47*Inputs!$B$29)</f>
+        <v>1.34927410581817</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2778,8 +2785,8 @@
         <v>120</v>
       </c>
       <c r="B31" s="10" t="n">
-        <f aca="false">MAX(0,(B27*Inputs!$B$32-Inputs!$B$19)*Inputs!$B$12)</f>
-        <v>1407938.68378812</v>
+        <f aca="false">MAX(0,(Inputs!$B$47*Inputs!$B$29-Inputs!$B$19)*Inputs!$B$12)</f>
+        <v>2622643.65971108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Roehampton: base case purchase price £18m
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -39,7 +39,7 @@
     <t xml:space="preserve">£m</t>
   </si>
   <si>
-    <t xml:space="preserve">Working price; no guide published. The appraisal page gives the bid for 15% on cost with the residential placeholder at £7m. Use Goal Seek on Outputs, Profit on cost, by changing this cell.</t>
+    <t xml:space="preserve">Base case; no guide published. The appraisal page gives the bid for 15% on cost with the residential placeholder at £7m. Use Goal Seek on Outputs, Profit on cost, by changing this cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Purchaser's costs</t>
@@ -895,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>4</v>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B38" s="10" t="n">
         <f aca="false">Inputs!$B$5*1000000</f>
-        <v>30000000</v>
+        <v>18000000</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B46" s="10" t="n">
         <f aca="false">B38*(1+Inputs!$B$6)+B36+Inputs!$B$20</f>
-        <v>33844260</v>
+        <v>21028260</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="G5" s="10" t="n">
         <f aca="false">-C5*(IF(A5=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$34+Inputs!$B$35,0))</f>
-        <v>-33844260</v>
+        <v>-21028260</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">-C5*IF(AND(Inputs!$B$24&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
@@ -1585,11 +1585,11 @@
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">SUM(D5:I5)</f>
-        <v>-33844260</v>
+        <v>-21028260</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">-G5-F5</f>
-        <v>33844260</v>
+        <v>21028260</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF(A5=0,Inputs!$B$47,0)</f>
@@ -1621,11 +1621,11 @@
       </c>
       <c r="S5" s="10" t="n">
         <f aca="false">J5+R5</f>
-        <v>-18398126.6399144</v>
+        <v>-5582126.63991439</v>
       </c>
       <c r="T5" s="10" t="n">
         <f aca="false">S5</f>
-        <v>-18398126.6399144</v>
+        <v>-5582126.63991439</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">T5+S6</f>
-        <v>-19709448.4697699</v>
+        <v>-6893448.46976993</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="T7" s="10" t="n">
         <f aca="false">T6+S7</f>
-        <v>-21020770.2996255</v>
+        <v>-8204770.29962547</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="T8" s="10" t="n">
         <f aca="false">T7+S8</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="T9" s="10" t="n">
         <f aca="false">T8+S9</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="T10" s="10" t="n">
         <f aca="false">T9+S10</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="T11" s="10" t="n">
         <f aca="false">T10+S11</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">T11+S12</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="T13" s="10" t="n">
         <f aca="false">T12+S13</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="T14" s="10" t="n">
         <f aca="false">T13+S14</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="T15" s="10" t="n">
         <f aca="false">T14+S15</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">SUM(G5:G15)</f>
-        <v>-33844260</v>
+        <v>-21028260</v>
       </c>
       <c r="H16" s="14" t="n">
         <f aca="false">SUM(H5:H15)</f>
@@ -2470,11 +2470,11 @@
       </c>
       <c r="J16" s="14" t="n">
         <f aca="false">SUM(J5:J15)</f>
-        <v>-377292.669876941</v>
+        <v>12438707.3301231</v>
       </c>
       <c r="K16" s="14" t="n">
         <f aca="false">SUM(K5:K15)</f>
-        <v>26844260</v>
+        <v>14028260</v>
       </c>
       <c r="L16" s="14" t="n">
         <f aca="false">SUM(L5:L15)</f>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="S16" s="14" t="n">
         <f aca="false">SUM(S5:S15)</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
       <c r="T16" s="2"/>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">-'Cash flow'!G16-'Cash flow'!H16</f>
-        <v>33844260</v>
+        <v>21028260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">B10+B11</f>
-        <v>38313445.7945425</v>
+        <v>25497445.7945425</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="B13" s="15" t="n">
         <f aca="false">(B8-B12)/B12</f>
-        <v>-0.126495499527997</v>
+        <v>0.312561564001298</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">B8-B12</f>
-        <v>-4846478.46441948</v>
+        <v>7969521.53558052</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="B16" s="15" t="n">
         <f aca="false">B15/B8</f>
-        <v>-0.144813792555899</v>
+        <v>0.238130974251954</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">(Inputs!$B$33+Inputs!$B$19)/(B10-Inputs!$B$39)</f>
-        <v>0.07093732514884</v>
+        <v>0.135744561335476</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">IRR('Cash flow'!J5:J15,-0.05)</f>
-        <v>-0.00374098634422967</v>
+        <v>0.168157145213216</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B19" s="15" t="n">
         <f aca="false">IRR('Cash flow'!S5:S15,-0.2)</f>
-        <v>-0.0893772076578962</v>
+        <v>0.299682183075168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
-        <v>0.769443346017352</v>
+        <v>1.97132780620858</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">-MIN('Cash flow'!T5:T15)</f>
-        <v>21020770.2996255</v>
+        <v>8204770.29962547</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">(Inputs!$B$33+Inputs!$B$19-B22*Inputs!$B$29)/B21</f>
-        <v>0.0234500526440387</v>
+        <v>0.0600794601363751</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B27" s="15" t="n">
         <f aca="false">Inputs!$B$47/Inputs!$B$46</f>
-        <v>0.463338647825703</v>
+        <v>0.745727590635722</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="B28" s="10" t="n">
         <f aca="false">Inputs!$B$46-Inputs!$B$47</f>
-        <v>18162906.3349385</v>
+        <v>5346906.33493847</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Roehampton: The Grange and cottages at BGP's £7m exit valuation, not a placeholder
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -159,10 +159,10 @@
     <t xml:space="preserve">Grange holding cost until sold: 0 while Related's underwrite carries the conversion costs and value; c. £1,000,000 pa if held empty</t>
   </si>
   <si>
-    <t xml:space="preserve">The Grange and cottages, placeholder value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder value for The Grange and the cottages together, pending Related's residential underwrite (Woody Bruce, 17 October 2026)</t>
+    <t xml:space="preserve">The Grange and cottages, exit valuation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BGP's exit valuation of The Grange and the cottages together, sold with everything else at the end of the hold; Related are underwriting the conversion</t>
   </si>
   <si>
     <t xml:space="preserve">Debt</t>
@@ -342,7 +342,7 @@
     <t xml:space="preserve">Profit on receipts</t>
   </si>
   <si>
-    <t xml:space="preserve">Yield on cost, stabilised rent over cost net of the residential placeholder</t>
+    <t xml:space="preserve">Yield on cost, stabilised rent over cost net of the residential value</t>
   </si>
   <si>
     <t xml:space="preserve">Unlevered IRR</t>

</xml_diff>

<commit_message>
Roehampton: Grange exit valuation fixed at £7m, drop the breakeven against the bid
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -39,7 +39,7 @@
     <t xml:space="preserve">£m</t>
   </si>
   <si>
-    <t xml:space="preserve">Base case; no guide published. The appraisal page gives the bid for 15% on cost with the residential placeholder at £7m. Use Goal Seek on Outputs, Profit on cost, by changing this cell.</t>
+    <t xml:space="preserve">Base case; no guide published. The appraisal page gives the bid for 15% on cost with The Grange and cottages at BGP's £7m exit valuation. Use Goal Seek on Outputs, Profit on cost, by changing this cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Purchaser's costs</t>
@@ -303,7 +303,7 @@
     <t xml:space="preserve">Outputs</t>
   </si>
   <si>
-    <t xml:space="preserve">All figures recompute from Inputs. For the breakeven bid, Goal Seek Outputs!B13 to the target by changing the purchase price on Inputs; for the residential breakeven, change the Grange and cottages placeholder instead.</t>
+    <t xml:space="preserve">All figures recompute from Inputs. For the breakeven bid, Goal Seek Outputs!B13 to the target by changing the purchase price on Inputs.</t>
   </si>
   <si>
     <t xml:space="preserve">Receipts</t>

</xml_diff>

<commit_message>
Roehampton: base case on Nick's observations and the Lighthouse survey; developer's shell works, 2 years capital, 1 year rent free; arrival area; HoTs with alienation
</commit_message>
<xml_diff>
--- a/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
+++ b/client/public/share/roehampton-sports-ground-estate-k7x2/docs/Roehampton - Underwrite model - BGP.xlsx
@@ -105,7 +105,7 @@
     <t xml:space="preserve">£ psf</t>
   </si>
   <si>
-    <t xml:space="preserve">Nil: Third Space fit out from the capital contribution and nothing more is spent on the leisure side</t>
+    <t xml:space="preserve">Developer's shell before the lease: roofs, glazing, cladding and fabric per the Lighthouse 2019 survey (£5.5m on the two buildings at 2019 prices), inflated, plus strip-out and the new link; M&amp;E left to the tenant's fit-out; pending a QS (Nick, 19 Oct 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Fees and contingency on works</t>
@@ -234,7 +234,7 @@
     <t xml:space="preserve">Annual cash flow, £</t>
   </si>
   <si>
-    <t xml:space="preserve">Completion January 2027 (year 0): purchase, Third Space lease, capital contribution and the Club's surrender and regrant all on the same day. Nothing more spent on the leisure side; everything sold as one lot at the end of the hold year. Rows beyond the hold year are zero.</t>
+    <t xml:space="preserve">Completion January 2027 (year 0): purchase and the Club's surrender and regrant; agreement for lease with Third Space. 2027 (year 1): landlord's works to developer's shell, then the lease with the capital contribution on handover; rent free from the lease start. Everything sold as one lot at the end of the hold year. Rows beyond the hold year are zero.</t>
   </si>
   <si>
     <t xml:space="preserve">Year</t>
@@ -983,7 +983,7 @@
         <v>19</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>10</v>
@@ -995,7 +995,7 @@
         <v>20</v>
       </c>
       <c r="B13" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>21</v>
@@ -1021,7 +1021,7 @@
         <v>25</v>
       </c>
       <c r="B15" s="8" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>26</v>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$15</f>
-        <v>0</v>
+        <v>7818460</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">B34*Inputs!$B$16</f>
-        <v>0</v>
+        <v>1172769</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">B33*Inputs!$B$13</f>
-        <v>1804260</v>
+        <v>3608520</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B37" s="10" t="n">
         <f aca="false">B33*Inputs!$B$12</f>
-        <v>3608520</v>
+        <v>1804260</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -1374,8 +1374,8 @@
         <v>67</v>
       </c>
       <c r="B46" s="10" t="n">
-        <f aca="false">B38*(1+Inputs!$B$6)+B36+Inputs!$B$20</f>
-        <v>21028260</v>
+        <f aca="false">B38*(1+Inputs!$B$6)+Inputs!$B$20</f>
+        <v>19224000</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -1572,8 +1572,8 @@
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <f aca="false">-C5*(IF(A5=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$34+Inputs!$B$35,0))</f>
-        <v>-21028260</v>
+        <f aca="false">-C5*(IF(A5=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A5=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
+        <v>-19224000</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">-C5*IF(AND(Inputs!$B$24&gt;0,A5&gt;=1,A5&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
@@ -1585,11 +1585,11 @@
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">SUM(D5:I5)</f>
-        <v>-21028260</v>
+        <v>-19224000</v>
       </c>
       <c r="K5" s="10" t="n">
         <f aca="false">-G5-F5</f>
-        <v>21028260</v>
+        <v>19224000</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF(A5=0,Inputs!$B$47,0)</f>
@@ -1621,11 +1621,11 @@
       </c>
       <c r="S5" s="10" t="n">
         <f aca="false">J5+R5</f>
-        <v>-5582126.63991439</v>
+        <v>-3777866.63991439</v>
       </c>
       <c r="T5" s="10" t="n">
         <f aca="false">S5</f>
-        <v>-5582126.63991439</v>
+        <v>-3777866.63991439</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1653,8 +1653,8 @@
         <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">-C6*(IF(A6=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A6=1,Inputs!$B$34+Inputs!$B$35,0))</f>
-        <v>-0</v>
+        <f aca="false">-C6*(IF(A6=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A6=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
+        <v>-12599749</v>
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">-C6*IF(AND(Inputs!$B$24&gt;0,A6&gt;=1,A6&lt;=Inputs!$B$24),Inputs!$B$25,0)</f>
@@ -1666,11 +1666,11 @@
       </c>
       <c r="J6" s="10" t="n">
         <f aca="false">SUM(D6:I6)</f>
-        <v>100000</v>
+        <v>-12499749</v>
       </c>
       <c r="K6" s="10" t="n">
         <f aca="false">-G6-F6</f>
-        <v>0</v>
+        <v>12599749</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF(A6=0,Inputs!$B$47,0)</f>
@@ -1702,11 +1702,11 @@
       </c>
       <c r="S6" s="10" t="n">
         <f aca="false">J6+R6</f>
-        <v>-1311321.82985554</v>
+        <v>-13911070.8298555</v>
       </c>
       <c r="T6" s="10" t="n">
         <f aca="false">T5+S6</f>
-        <v>-6893448.46976993</v>
+        <v>-17688937.4697699</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1727,14 +1727,14 @@
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">C7*IF(A7&lt;1,0,IF(A7&lt;=Inputs!$B$12,0,IF(A7-1&lt;Inputs!$B$12,A7-Inputs!$B$12,1)*Inputs!$B$33*(1+Inputs!$B$14)^(5*INT((A7-1)/5))))</f>
-        <v>0</v>
+        <v>1804260</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">C7*(IF(A7=0,IF(Inputs!$B$24=0,Inputs!$B$39,0),0)+IF(AND(Inputs!$B$24&gt;0,A7=Inputs!$B$24),Inputs!$B$39,0))</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
-        <f aca="false">-C7*(IF(A7=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A7=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C7*(IF(A7=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A7=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H7" s="10" t="n">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="J7" s="10" t="n">
         <f aca="false">SUM(D7:I7)</f>
-        <v>100000</v>
+        <v>1904260</v>
       </c>
       <c r="K7" s="10" t="n">
         <f aca="false">-G7-F7</f>
@@ -1783,11 +1783,11 @@
       </c>
       <c r="S7" s="10" t="n">
         <f aca="false">J7+R7</f>
-        <v>-1311321.82985554</v>
+        <v>492938.170144463</v>
       </c>
       <c r="T7" s="10" t="n">
         <f aca="false">T6+S7</f>
-        <v>-8204770.29962547</v>
+        <v>-17195999.2996255</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1815,7 +1815,7 @@
         <v>7000000</v>
       </c>
       <c r="G8" s="10" t="n">
-        <f aca="false">-C8*(IF(A8=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A8=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C8*(IF(A8=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A8=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H8" s="10" t="n">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="T8" s="10" t="n">
         <f aca="false">T7+S8</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1896,7 +1896,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
-        <f aca="false">-C9*(IF(A9=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A9=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C9*(IF(A9=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A9=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H9" s="10" t="n">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="T9" s="10" t="n">
         <f aca="false">T8+S9</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
-        <f aca="false">-C10*(IF(A10=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A10=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C10*(IF(A10=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A10=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H10" s="10" t="n">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="T10" s="10" t="n">
         <f aca="false">T9+S10</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2058,7 +2058,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <f aca="false">-C11*(IF(A11=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A11=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C11*(IF(A11=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A11=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H11" s="10" t="n">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="T11" s="10" t="n">
         <f aca="false">T10+S11</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2139,7 +2139,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
-        <f aca="false">-C12*(IF(A12=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A12=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C12*(IF(A12=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A12=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H12" s="10" t="n">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="T12" s="10" t="n">
         <f aca="false">T11+S12</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
-        <f aca="false">-C13*(IF(A13=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A13=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C13*(IF(A13=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A13=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H13" s="10" t="n">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="T13" s="10" t="n">
         <f aca="false">T12+S13</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
-        <f aca="false">-C14*(IF(A14=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A14=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C14*(IF(A14=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A14=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H14" s="10" t="n">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="T14" s="10" t="n">
         <f aca="false">T13+S14</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2382,7 +2382,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="10" t="n">
-        <f aca="false">-C15*(IF(A15=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$36+Inputs!$B$20,0)+IF(A15=1,Inputs!$B$34+Inputs!$B$35,0))</f>
+        <f aca="false">-C15*(IF(A15=0,Inputs!$B$38*(1+Inputs!$B$6)+Inputs!$B$20,0)+IF(A15=1,Inputs!$B$34+Inputs!$B$35+Inputs!$B$36,0))</f>
         <v>-0</v>
       </c>
       <c r="H15" s="10" t="n">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="T15" s="10" t="n">
         <f aca="false">T14+S15</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">SUM(E5:E15)</f>
-        <v>1804260</v>
+        <v>3608520</v>
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">SUM(F5:F15)</f>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">SUM(G5:G15)</f>
-        <v>-21028260</v>
+        <v>-31823749</v>
       </c>
       <c r="H16" s="14" t="n">
         <f aca="false">SUM(H5:H15)</f>
@@ -2470,11 +2470,11 @@
       </c>
       <c r="J16" s="14" t="n">
         <f aca="false">SUM(J5:J15)</f>
-        <v>12438707.3301231</v>
+        <v>3447478.33012306</v>
       </c>
       <c r="K16" s="14" t="n">
         <f aca="false">SUM(K5:K15)</f>
-        <v>14028260</v>
+        <v>24823749</v>
       </c>
       <c r="L16" s="14" t="n">
         <f aca="false">SUM(L5:L15)</f>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="S16" s="14" t="n">
         <f aca="false">SUM(S5:S15)</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
       <c r="T16" s="2"/>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">'Cash flow'!D16+'Cash flow'!E16</f>
-        <v>2104260</v>
+        <v>3908520</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B8" s="10" t="n">
         <f aca="false">B5+B6+B7</f>
-        <v>33466967.3301231</v>
+        <v>35271227.3301231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">-'Cash flow'!G16-'Cash flow'!H16</f>
-        <v>21028260</v>
+        <v>31823749</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">B10+B11</f>
-        <v>25497445.7945425</v>
+        <v>36292934.7945425</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="B13" s="15" t="n">
         <f aca="false">(B8-B12)/B12</f>
-        <v>0.312561564001298</v>
+        <v>-0.0281516904103637</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">B8-B12</f>
-        <v>7969521.53558052</v>
+        <v>-1021707.46441948</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="B16" s="15" t="n">
         <f aca="false">B15/B8</f>
-        <v>0.238130974251954</v>
+        <v>-0.028967165073581</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">(Inputs!$B$33+Inputs!$B$19)/(B10-Inputs!$B$39)</f>
-        <v>0.135744561335476</v>
+        <v>0.0767112171493516</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">IRR('Cash flow'!J5:J15,-0.05)</f>
-        <v>0.168157145213216</v>
+        <v>0.0411932065521182</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B19" s="15" t="n">
         <f aca="false">IRR('Cash flow'!S5:S15,-0.2)</f>
-        <v>0.299682183075168</v>
+        <v>-0.026896564523716</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">SUMIF('Cash flow'!S5:S15,"&gt;0")/-SUMIF('Cash flow'!S5:S15,"&lt;0")</f>
-        <v>1.97132780620858</v>
+        <v>0.942240314537515</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">-MIN('Cash flow'!T5:T15)</f>
-        <v>8204770.29962547</v>
+        <v>17688937.4697699</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">(Inputs!$B$33+Inputs!$B$19-B22*Inputs!$B$29)/B21</f>
-        <v>0.0600794601363751</v>
+        <v>0.0278670310744715</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B27" s="15" t="n">
         <f aca="false">Inputs!$B$47/Inputs!$B$46</f>
-        <v>0.745727590635722</v>
+        <v>0.815717523151349</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="B28" s="10" t="n">
         <f aca="false">Inputs!$B$46-Inputs!$B$47</f>
-        <v>5346906.33493847</v>
+        <v>3542646.33493847</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B31" s="10" t="n">
         <f aca="false">MAX(0,(Inputs!$B$47*Inputs!$B$29-Inputs!$B$19)*Inputs!$B$12)</f>
-        <v>2622643.65971108</v>
+        <v>1311321.82985554</v>
       </c>
     </row>
   </sheetData>

</xml_diff>